<commit_message>
Leadership deck v3: Feasibility -> Cost x3 -> Logistics + PCI question -> Decision
- Binary decision: second source = max(1/3 of demand, 1 drum/week) or nothing;
  no warm-backup option (suppliers require >=1 drum/week)
- New upside slide: price below $2.50/lb and the opportunity cost of not looking
- Full supplier names throughout; speaker notes on every slide
- Model: effective-share logic, upside sensitivity rows

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
@@ -20,18 +20,20 @@
     <definedName name="LbWk">Inputs!$C$8</definedName>
     <definedName name="Weeks">Inputs!$C$9</definedName>
     <definedName name="Growth">Inputs!$C$10</definedName>
-    <definedName name="Share">Inputs!$C$11</definedName>
-    <definedName name="WarmShare">Inputs!$C$12</definedName>
-    <definedName name="PCIlo">Inputs!$C$13</definedName>
-    <definedName name="PCImid">Inputs!$C$14</definedName>
-    <definedName name="PCIhi">Inputs!$C$15</definedName>
-    <definedName name="MktLo">Inputs!$C$16</definedName>
-    <definedName name="MktBase">Inputs!$C$17</definedName>
-    <definedName name="MktHi">Inputs!$C$18</definedName>
-    <definedName name="CJBlb">Inputs!$C$19</definedName>
-    <definedName name="QualCost">Inputs!$C$20</definedName>
-    <definedName name="Pdis">Inputs!$C$21</definedName>
-    <definedName name="Dcost">Inputs!$C$22</definedName>
+    <definedName name="MinDrumsWk">Inputs!$C$11</definedName>
+    <definedName name="MinShare">Inputs!$C$12</definedName>
+    <definedName name="Share">Inputs!$C$13</definedName>
+    <definedName name="EffShare">Inputs!$C$14</definedName>
+    <definedName name="PCIlo">Inputs!$C$15</definedName>
+    <definedName name="PCImid">Inputs!$C$16</definedName>
+    <definedName name="PCIhi">Inputs!$C$17</definedName>
+    <definedName name="MktLo">Inputs!$C$18</definedName>
+    <definedName name="MktBase">Inputs!$C$19</definedName>
+    <definedName name="MktHi">Inputs!$C$20</definedName>
+    <definedName name="CJBlb">Inputs!$C$21</definedName>
+    <definedName name="QualCost">Inputs!$C$22</definedName>
+    <definedName name="Pdis">Inputs!$C$23</definedName>
+    <definedName name="Dcost">Inputs!$C$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -45,7 +47,7 @@
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="167" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,8 +89,14 @@
       <color rgb="00595959"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -113,6 +121,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D6DCE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -142,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,10 +166,13 @@
     <xf numFmtId="3" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -167,6 +183,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -538,12 +558,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D22"/>
+  <dimension ref="B2:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -556,7 +576,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Yellow = editable. Everything else recalculates. Define acronyms: PVA = polyvinyl alcohol; SNP = incumbent supplier; PCI = candidate second source.</t>
+          <t>Yellow = editable. PVA = polyvinyl alcohol. SNP Inc. = incumbent. PCI Manufacturing = candidate second source. The second source gets the LARGER of 1/3 of demand and its 1-drum/week minimum — or nothing.</t>
         </is>
       </c>
     </row>
@@ -588,14 +608,14 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Confirmed (SNP: 1/450-lb drum)</t>
+          <t>Confirmed (SNP Inc.: 1/450-lb drum)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>SNP price ($/lb delivered, all-in)</t>
+          <t>SNP Inc. price ($/lb delivered, all-in)</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
@@ -603,7 +623,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Real quote — SNP Est 012726-1</t>
+          <t>Real quote — SNP Estimate 012726-1</t>
         </is>
       </c>
     </row>
@@ -651,178 +671,210 @@
     <row r="11">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Share of volume to 2nd source (Option A)</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>0.3333333333333333</v>
+          <t>Smallest volume a second source will accept (drums/week)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>One-third of business</t>
+          <t>Supplier condition — below this they will not engage</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Share for a 'warm' backup (Option C)</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>0.05</v>
+          <t xml:space="preserve">  = share of today's demand</t>
+        </is>
+      </c>
+      <c r="C12" s="8">
+        <f>MinDrumsWk*DrumLb/LbWk</f>
+        <v/>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>~1 drum every 7 weeks</t>
+          <t>~35%. This is the smallest insurance available.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>PCI price — LOW ($/lb)</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>2.5</v>
+          <t>Target share of demand (Option A)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>0.3333333333333333</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Forecast floor</t>
+          <t>One-third. Year 1: 1/3 = 0.96 drums/wk, so the minimum (1.0) governs; from Year 2 the 1/3 governs.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>PCI price — MID ($/lb)</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>3.75</v>
+          <t xml:space="preserve">  = effective share, Year 1</t>
+        </is>
+      </c>
+      <c r="C14" s="8">
+        <f>MAX(Share,MinShare)</f>
+        <v/>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Midpoint of range</t>
+          <t>max(target, minimum)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>PCI price — HIGH ($/lb)</t>
+          <t>PCI price — LOW ($/lb)</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Forecast ceiling</t>
+          <t>Forecast floor</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Market reference — LOW ($/lb)</t>
+          <t>PCI price — MID ($/lb)</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>0.85</v>
+        <v>3.75</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Triangulated (resin floor + labor bottom-up)</t>
+          <t>Midpoint of range</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Market reference — BASE ($/lb)</t>
+          <t>PCI price — HIGH ($/lb)</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>1.4</v>
+        <v>5</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Triangulated</t>
+          <t>Forecast ceiling</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Market reference — HIGH ($/lb)</t>
+          <t>Market reference — LOW ($/lb)</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>2.55</v>
+        <v>0.85</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Triangulated (retail ceiling)</t>
+          <t>Triangulated (resin floor + labor bottom-up)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>CJB quote, landed ($/lb) — reference only</t>
+          <t>Market reference — BASE ($/lb)</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>8.42</v>
+        <v>1.4</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>$8-8.50 toll excl. materials + $75/drum resin; ~11x SNP</t>
+          <t>Triangulated</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>One-time qualification cost ($)</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="n">
-        <v>15000</v>
+          <t>Market reference — HIGH ($/lb)</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>2.55</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>PLACEHOLDER — engineering hrs, samples, hydrogel tests, SQA, audit. Confirm.</t>
+          <t>Triangulated (retail ceiling)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Disruption probability per year (for break-even)</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>0.05</v>
+          <t>CJB Applied Technologies quote, landed ($/lb) — reference</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>8.42</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>PLACEHOLDER — leadership judgement</t>
+          <t>$8-8.50 toll excl. materials + $75/drum resin; ~11x SNP</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Cost of a 6-month SNP outage ($)</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="n">
+          <t>One-time qualification cost ($)</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER — engineering hrs, samples, hydrogel tests, quality agreement. Confirm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Disruption probability per year (for break-even)</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER — leadership judgement</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Cost of a 6-month SNP Inc. outage ($)</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="n">
         <v>500000</v>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>PLACEHOLDER — revenue at risk + expedite + line-down. NEEDED FROM FINANCE/OPS.</t>
         </is>
@@ -839,32 +891,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K13"/>
+  <dimension ref="B2:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Five-year cost of Option A (dual-source at the chosen share)</t>
+          <t>Five-year cost of Option A</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Premium = share x (PCI price - SNP price) x annual lb. It scales 1:1 with volume, so growth compounds it.</t>
+          <t>Each year the second source gets max(1/3 of demand, 1 drum/week). Premium = share x (PCI price - SNP price) x annual lb; it grows with volume.</t>
         </is>
       </c>
     </row>
@@ -886,295 +940,345 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
+          <t>Effective share</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Drums/wk to PCI</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
           <t>All-SNP baseline</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Option A @ PCI LOW</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Option A @ PCI MID</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Option A @ PCI HIGH</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Premium LOW</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Premium MID</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>Premium HIGH</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="12">
         <f>LbWk*Weeks*(1+Growth)^(1-1)</f>
         <v/>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="12">
         <f>C6/DrumLb</f>
         <v/>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="13">
+        <f>MAX(Share,MinDrumsWk*Weeks*DrumLb/C6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="14">
+        <f>D6*E6/Weeks</f>
+        <v/>
+      </c>
+      <c r="G6" s="15">
         <f>C6*SNPlb</f>
         <v/>
       </c>
-      <c r="F6" s="12">
-        <f>C6*(1-Share)*SNPlb+C6*Share*PCIlo</f>
-        <v/>
-      </c>
-      <c r="G6" s="12">
-        <f>C6*(1-Share)*SNPlb+C6*Share*PCImid</f>
-        <v/>
-      </c>
-      <c r="H6" s="12">
-        <f>C6*(1-Share)*SNPlb+C6*Share*PCIhi</f>
-        <v/>
-      </c>
-      <c r="I6" s="13">
-        <f>F6-E6</f>
-        <v/>
-      </c>
-      <c r="J6" s="13">
-        <f>G6-E6</f>
-        <v/>
-      </c>
-      <c r="K6" s="13">
-        <f>H6-E6</f>
+      <c r="H6" s="15">
+        <f>C6*(1-E6)*SNPlb+C6*E6*PCIlo</f>
+        <v/>
+      </c>
+      <c r="I6" s="15">
+        <f>C6*(1-E6)*SNPlb+C6*E6*PCImid</f>
+        <v/>
+      </c>
+      <c r="J6" s="15">
+        <f>C6*(1-E6)*SNPlb+C6*E6*PCIhi</f>
+        <v/>
+      </c>
+      <c r="K6" s="16">
+        <f>H6-G6</f>
+        <v/>
+      </c>
+      <c r="L6" s="16">
+        <f>I6-G6</f>
+        <v/>
+      </c>
+      <c r="M6" s="16">
+        <f>J6-G6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="12">
         <f>LbWk*Weeks*(1+Growth)^(2-1)</f>
         <v/>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="12">
         <f>C7/DrumLb</f>
         <v/>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="13">
+        <f>MAX(Share,MinDrumsWk*Weeks*DrumLb/C7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="14">
+        <f>D7*E7/Weeks</f>
+        <v/>
+      </c>
+      <c r="G7" s="15">
         <f>C7*SNPlb</f>
         <v/>
       </c>
-      <c r="F7" s="12">
-        <f>C7*(1-Share)*SNPlb+C7*Share*PCIlo</f>
-        <v/>
-      </c>
-      <c r="G7" s="12">
-        <f>C7*(1-Share)*SNPlb+C7*Share*PCImid</f>
-        <v/>
-      </c>
-      <c r="H7" s="12">
-        <f>C7*(1-Share)*SNPlb+C7*Share*PCIhi</f>
-        <v/>
-      </c>
-      <c r="I7" s="13">
-        <f>F7-E7</f>
-        <v/>
-      </c>
-      <c r="J7" s="13">
-        <f>G7-E7</f>
-        <v/>
-      </c>
-      <c r="K7" s="13">
-        <f>H7-E7</f>
+      <c r="H7" s="15">
+        <f>C7*(1-E7)*SNPlb+C7*E7*PCIlo</f>
+        <v/>
+      </c>
+      <c r="I7" s="15">
+        <f>C7*(1-E7)*SNPlb+C7*E7*PCImid</f>
+        <v/>
+      </c>
+      <c r="J7" s="15">
+        <f>C7*(1-E7)*SNPlb+C7*E7*PCIhi</f>
+        <v/>
+      </c>
+      <c r="K7" s="16">
+        <f>H7-G7</f>
+        <v/>
+      </c>
+      <c r="L7" s="16">
+        <f>I7-G7</f>
+        <v/>
+      </c>
+      <c r="M7" s="16">
+        <f>J7-G7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="12">
         <f>LbWk*Weeks*(1+Growth)^(3-1)</f>
         <v/>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="12">
         <f>C8/DrumLb</f>
         <v/>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="13">
+        <f>MAX(Share,MinDrumsWk*Weeks*DrumLb/C8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="14">
+        <f>D8*E8/Weeks</f>
+        <v/>
+      </c>
+      <c r="G8" s="15">
         <f>C8*SNPlb</f>
         <v/>
       </c>
-      <c r="F8" s="12">
-        <f>C8*(1-Share)*SNPlb+C8*Share*PCIlo</f>
-        <v/>
-      </c>
-      <c r="G8" s="12">
-        <f>C8*(1-Share)*SNPlb+C8*Share*PCImid</f>
-        <v/>
-      </c>
-      <c r="H8" s="12">
-        <f>C8*(1-Share)*SNPlb+C8*Share*PCIhi</f>
-        <v/>
-      </c>
-      <c r="I8" s="13">
-        <f>F8-E8</f>
-        <v/>
-      </c>
-      <c r="J8" s="13">
-        <f>G8-E8</f>
-        <v/>
-      </c>
-      <c r="K8" s="13">
-        <f>H8-E8</f>
+      <c r="H8" s="15">
+        <f>C8*(1-E8)*SNPlb+C8*E8*PCIlo</f>
+        <v/>
+      </c>
+      <c r="I8" s="15">
+        <f>C8*(1-E8)*SNPlb+C8*E8*PCImid</f>
+        <v/>
+      </c>
+      <c r="J8" s="15">
+        <f>C8*(1-E8)*SNPlb+C8*E8*PCIhi</f>
+        <v/>
+      </c>
+      <c r="K8" s="16">
+        <f>H8-G8</f>
+        <v/>
+      </c>
+      <c r="L8" s="16">
+        <f>I8-G8</f>
+        <v/>
+      </c>
+      <c r="M8" s="16">
+        <f>J8-G8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="12">
         <f>LbWk*Weeks*(1+Growth)^(4-1)</f>
         <v/>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="12">
         <f>C9/DrumLb</f>
         <v/>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="13">
+        <f>MAX(Share,MinDrumsWk*Weeks*DrumLb/C9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="14">
+        <f>D9*E9/Weeks</f>
+        <v/>
+      </c>
+      <c r="G9" s="15">
         <f>C9*SNPlb</f>
         <v/>
       </c>
-      <c r="F9" s="12">
-        <f>C9*(1-Share)*SNPlb+C9*Share*PCIlo</f>
-        <v/>
-      </c>
-      <c r="G9" s="12">
-        <f>C9*(1-Share)*SNPlb+C9*Share*PCImid</f>
-        <v/>
-      </c>
-      <c r="H9" s="12">
-        <f>C9*(1-Share)*SNPlb+C9*Share*PCIhi</f>
-        <v/>
-      </c>
-      <c r="I9" s="13">
-        <f>F9-E9</f>
-        <v/>
-      </c>
-      <c r="J9" s="13">
-        <f>G9-E9</f>
-        <v/>
-      </c>
-      <c r="K9" s="13">
-        <f>H9-E9</f>
+      <c r="H9" s="15">
+        <f>C9*(1-E9)*SNPlb+C9*E9*PCIlo</f>
+        <v/>
+      </c>
+      <c r="I9" s="15">
+        <f>C9*(1-E9)*SNPlb+C9*E9*PCImid</f>
+        <v/>
+      </c>
+      <c r="J9" s="15">
+        <f>C9*(1-E9)*SNPlb+C9*E9*PCIhi</f>
+        <v/>
+      </c>
+      <c r="K9" s="16">
+        <f>H9-G9</f>
+        <v/>
+      </c>
+      <c r="L9" s="16">
+        <f>I9-G9</f>
+        <v/>
+      </c>
+      <c r="M9" s="16">
+        <f>J9-G9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="12">
         <f>LbWk*Weeks*(1+Growth)^(5-1)</f>
         <v/>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="12">
         <f>C10/DrumLb</f>
         <v/>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="13">
+        <f>MAX(Share,MinDrumsWk*Weeks*DrumLb/C10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="14">
+        <f>D10*E10/Weeks</f>
+        <v/>
+      </c>
+      <c r="G10" s="15">
         <f>C10*SNPlb</f>
         <v/>
       </c>
-      <c r="F10" s="12">
-        <f>C10*(1-Share)*SNPlb+C10*Share*PCIlo</f>
-        <v/>
-      </c>
-      <c r="G10" s="12">
-        <f>C10*(1-Share)*SNPlb+C10*Share*PCImid</f>
-        <v/>
-      </c>
-      <c r="H10" s="12">
-        <f>C10*(1-Share)*SNPlb+C10*Share*PCIhi</f>
-        <v/>
-      </c>
-      <c r="I10" s="13">
-        <f>F10-E10</f>
-        <v/>
-      </c>
-      <c r="J10" s="13">
-        <f>G10-E10</f>
-        <v/>
-      </c>
-      <c r="K10" s="13">
-        <f>H10-E10</f>
+      <c r="H10" s="15">
+        <f>C10*(1-E10)*SNPlb+C10*E10*PCIlo</f>
+        <v/>
+      </c>
+      <c r="I10" s="15">
+        <f>C10*(1-E10)*SNPlb+C10*E10*PCImid</f>
+        <v/>
+      </c>
+      <c r="J10" s="15">
+        <f>C10*(1-E10)*SNPlb+C10*E10*PCIhi</f>
+        <v/>
+      </c>
+      <c r="K10" s="16">
+        <f>H10-G10</f>
+        <v/>
+      </c>
+      <c r="L10" s="16">
+        <f>I10-G10</f>
+        <v/>
+      </c>
+      <c r="M10" s="16">
+        <f>J10-G10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>5-yr total</t>
         </is>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="18">
         <f>SUM(C6:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="18">
         <f>SUM(D6:D10)</f>
         <v/>
       </c>
-      <c r="E11" s="16">
-        <f>SUM(E6:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="16">
-        <f>SUM(F6:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="16">
+      <c r="G11" s="19">
         <f>SUM(G6:G10)</f>
         <v/>
       </c>
-      <c r="H11" s="16">
+      <c r="H11" s="19">
         <f>SUM(H6:H10)</f>
         <v/>
       </c>
-      <c r="I11" s="16">
+      <c r="I11" s="19">
         <f>SUM(I6:I10)</f>
         <v/>
       </c>
-      <c r="J11" s="16">
+      <c r="J11" s="19">
         <f>SUM(J6:J10)</f>
         <v/>
       </c>
-      <c r="K11" s="16">
+      <c r="K11" s="19">
         <f>SUM(K6:K10)</f>
+        <v/>
+      </c>
+      <c r="L11" s="19">
+        <f>SUM(L6:L10)</f>
+        <v/>
+      </c>
+      <c r="M11" s="19">
+        <f>SUM(M6:M10)</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Plus one-time qualification cost (Inputs) — applies to any second source, warm or active:</t>
-        </is>
-      </c>
-      <c r="E13" s="17">
+          <t>Plus one-time qualification cost (Inputs):</t>
+        </is>
+      </c>
+      <c r="G13" s="20">
         <f>QualCost</f>
         <v/>
       </c>
@@ -1190,27 +1294,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F23"/>
+  <dimension ref="B2:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>What drives the premium: 2nd-source price and share (Year 1)</t>
+          <t>What drives the premium (Year 1, at the supplier minimum ≈ 1/3)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Premium is linear in both. The share is the lever we control; the price is what the market gives us.</t>
+          <t>Price is what the market gives us. Share is NOT a free lever: anything below the supplier minimum is not available.</t>
         </is>
       </c>
     </row>
@@ -1227,377 +1330,332 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Premium @ 1/3 share</t>
+          <t>Premium (Year 1)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>x baseline</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Premium @ 5% (warm)</t>
+          <t>x today's PVA spend</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="18">
+      <c r="B6" s="21">
         <f>MktLo</f>
         <v/>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>Market LOW</t>
         </is>
       </c>
-      <c r="D6" s="12">
-        <f>LbWk*Weeks*Share*(B6-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E6" s="20">
+      <c r="D6" s="15">
+        <f>LbWk*Weeks*EffShare*(B6-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="E6" s="23">
         <f>D6/(LbWk*Weeks*SNPlb)</f>
         <v/>
       </c>
-      <c r="F6" s="12">
-        <f>LbWk*Weeks*WarmShare*(B6-SNPlb)</f>
-        <v/>
-      </c>
     </row>
     <row r="7">
-      <c r="B7" s="18">
+      <c r="B7" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>Upside case / assumed in July (low)</t>
+        </is>
+      </c>
+      <c r="D7" s="15">
+        <f>LbWk*Weeks*EffShare*(B7-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="E7" s="23">
+        <f>D7/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="21" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Upside case / assumed in July (high)</t>
+        </is>
+      </c>
+      <c r="D8" s="15">
+        <f>LbWk*Weeks*EffShare*(B8-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="E8" s="23">
+        <f>D8/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="21">
         <f>MktBase</f>
         <v/>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>Market BASE</t>
         </is>
       </c>
-      <c r="D7" s="12">
-        <f>LbWk*Weeks*Share*(B7-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E7" s="20">
-        <f>D7/(LbWk*Weeks*SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F7" s="12">
-        <f>LbWk*Weeks*WarmShare*(B7-SNPlb)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>Told to leadership (low)</t>
-        </is>
-      </c>
-      <c r="D8" s="12">
-        <f>LbWk*Weeks*Share*(B8-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E8" s="20">
-        <f>D8/(LbWk*Weeks*SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F8" s="12">
-        <f>LbWk*Weeks*WarmShare*(B8-SNPlb)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="18" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="C9" s="19" t="inlineStr">
-        <is>
-          <t>Told to leadership (high)</t>
-        </is>
-      </c>
-      <c r="D9" s="12">
-        <f>LbWk*Weeks*Share*(B9-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E9" s="20">
+      <c r="D9" s="15">
+        <f>LbWk*Weeks*EffShare*(B9-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="E9" s="23">
         <f>D9/(LbWk*Weeks*SNPlb)</f>
         <v/>
       </c>
-      <c r="F9" s="12">
-        <f>LbWk*Weeks*WarmShare*(B9-SNPlb)</f>
-        <v/>
-      </c>
     </row>
     <row r="10">
-      <c r="B10" s="18">
+      <c r="B10" s="21" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>Upside case — trigger price</t>
+        </is>
+      </c>
+      <c r="D10" s="15">
+        <f>LbWk*Weeks*EffShare*(B10-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="E10" s="23">
+        <f>D10/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>Upside case — borderline</t>
+        </is>
+      </c>
+      <c r="D11" s="15">
+        <f>LbWk*Weeks*EffShare*(B11-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="E11" s="23">
+        <f>D11/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="21">
         <f>MktHi</f>
         <v/>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>Market HIGH</t>
         </is>
       </c>
-      <c r="D10" s="12">
-        <f>LbWk*Weeks*Share*(B10-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E10" s="20">
-        <f>D10/(LbWk*Weeks*SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F10" s="12">
-        <f>LbWk*Weeks*WarmShare*(B10-SNPlb)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="18">
+      <c r="D12" s="15">
+        <f>LbWk*Weeks*EffShare*(B12-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="E12" s="23">
+        <f>D12/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="21">
         <f>PCIlo</f>
         <v/>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>PCI LOW</t>
         </is>
       </c>
-      <c r="D11" s="12">
-        <f>LbWk*Weeks*Share*(B11-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E11" s="20">
-        <f>D11/(LbWk*Weeks*SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F11" s="12">
-        <f>LbWk*Weeks*WarmShare*(B11-SNPlb)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>PCI original assumption</t>
-        </is>
-      </c>
-      <c r="D12" s="12">
-        <f>LbWk*Weeks*Share*(B12-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E12" s="20">
-        <f>D12/(LbWk*Weeks*SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F12" s="12">
-        <f>LbWk*Weeks*WarmShare*(B12-SNPlb)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="18">
+      <c r="D13" s="15">
+        <f>LbWk*Weeks*EffShare*(B13-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="E13" s="23">
+        <f>D13/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="21">
         <f>PCImid</f>
         <v/>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>PCI MID</t>
         </is>
       </c>
-      <c r="D13" s="12">
-        <f>LbWk*Weeks*Share*(B13-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E13" s="20">
-        <f>D13/(LbWk*Weeks*SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F13" s="12">
-        <f>LbWk*Weeks*WarmShare*(B13-SNPlb)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="18">
+      <c r="D14" s="15">
+        <f>LbWk*Weeks*EffShare*(B14-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="E14" s="23">
+        <f>D14/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="21">
         <f>PCIhi</f>
         <v/>
       </c>
-      <c r="C14" s="19" t="inlineStr">
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>PCI HIGH</t>
         </is>
       </c>
-      <c r="D14" s="12">
-        <f>LbWk*Weeks*Share*(B14-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E14" s="20">
-        <f>D14/(LbWk*Weeks*SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F14" s="12">
-        <f>LbWk*Weeks*WarmShare*(B14-SNPlb)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="18">
+      <c r="D15" s="15">
+        <f>LbWk*Weeks*EffShare*(B15-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="E15" s="23">
+        <f>D15/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="21">
         <f>CJBlb</f>
         <v/>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>CJB quote (landed)</t>
         </is>
       </c>
-      <c r="D15" s="12">
-        <f>LbWk*Weeks*Share*(B15-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E15" s="20">
-        <f>D15/(LbWk*Weeks*SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F15" s="12">
-        <f>LbWk*Weeks*WarmShare*(B15-SNPlb)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="B18" s="3" t="inlineStr">
+      <c r="D16" s="15">
+        <f>LbWk*Weeks*EffShare*(B16-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>D16/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Share to 2nd source</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Drums/yr</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>Premium @ PCI LOW</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Drums/week</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Available?</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Premium @ PCI MID</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Premium @ PCI HIGH</t>
-        </is>
+    </row>
+    <row r="18">
+      <c r="B18" s="24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C18" s="14">
+        <f>LbWk*B18/DrumLb</f>
+        <v/>
+      </c>
+      <c r="D18" s="25">
+        <f>IF(C18&gt;=MinDrumsWk,"Yes",IF(B18&gt;=0.3,"Rounds up to the 1-drum minimum","NO — below supplier minimum"))</f>
+        <v/>
+      </c>
+      <c r="E18" s="26">
+        <f>IF(B18&gt;=0.3,LbWk*Weeks*MAX(B18,MinShare)*(PCImid-SNPlb),"n/a")</f>
+        <v/>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="21" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C19" s="11">
-        <f>LbWk*Weeks*B19/DrumLb</f>
-        <v/>
-      </c>
-      <c r="D19" s="12">
-        <f>LbWk*Weeks*B19*(PCIlo-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E19" s="12">
-        <f>LbWk*Weeks*B19*(PCImid-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F19" s="12">
-        <f>LbWk*Weeks*B19*(PCIhi-SNPlb)</f>
+      <c r="B19" s="24" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C19" s="14">
+        <f>LbWk*B19/DrumLb</f>
+        <v/>
+      </c>
+      <c r="D19" s="25">
+        <f>IF(C19&gt;=MinDrumsWk,"Yes",IF(B19&gt;=0.3,"Rounds up to the 1-drum minimum","NO — below supplier minimum"))</f>
+        <v/>
+      </c>
+      <c r="E19" s="26">
+        <f>IF(B19&gt;=0.3,LbWk*Weeks*MAX(B19,MinShare)*(PCImid-SNPlb),"n/a")</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="21" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C20" s="11">
-        <f>LbWk*Weeks*B20/DrumLb</f>
-        <v/>
-      </c>
-      <c r="D20" s="12">
-        <f>LbWk*Weeks*B20*(PCIlo-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E20" s="12">
-        <f>LbWk*Weeks*B20*(PCImid-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F20" s="12">
-        <f>LbWk*Weeks*B20*(PCIhi-SNPlb)</f>
+      <c r="B20" s="24" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C20" s="14">
+        <f>LbWk*B20/DrumLb</f>
+        <v/>
+      </c>
+      <c r="D20" s="25">
+        <f>IF(C20&gt;=MinDrumsWk,"Yes",IF(B20&gt;=0.3,"Rounds up to the 1-drum minimum","NO — below supplier minimum"))</f>
+        <v/>
+      </c>
+      <c r="E20" s="26">
+        <f>IF(B20&gt;=0.3,LbWk*Weeks*MAX(B20,MinShare)*(PCImid-SNPlb),"n/a")</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C21" s="11">
-        <f>LbWk*Weeks*B21/DrumLb</f>
-        <v/>
-      </c>
-      <c r="D21" s="12">
-        <f>LbWk*Weeks*B21*(PCIlo-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E21" s="12">
-        <f>LbWk*Weeks*B21*(PCImid-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F21" s="12">
-        <f>LbWk*Weeks*B21*(PCIhi-SNPlb)</f>
+      <c r="B21" s="24" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="C21" s="14">
+        <f>LbWk*B21/DrumLb</f>
+        <v/>
+      </c>
+      <c r="D21" s="27">
+        <f>IF(C21&gt;=MinDrumsWk,"Yes",IF(B21&gt;=0.3,"Rounds up to the 1-drum minimum","NO — below supplier minimum"))</f>
+        <v/>
+      </c>
+      <c r="E21" s="15">
+        <f>IF(B21&gt;=0.3,LbWk*Weeks*MAX(B21,MinShare)*(PCImid-SNPlb),"n/a")</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="21" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="C22" s="11">
-        <f>LbWk*Weeks*B22/DrumLb</f>
-        <v/>
-      </c>
-      <c r="D22" s="12">
-        <f>LbWk*Weeks*B22*(PCIlo-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E22" s="12">
-        <f>LbWk*Weeks*B22*(PCImid-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F22" s="12">
-        <f>LbWk*Weeks*B22*(PCIhi-SNPlb)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="21" t="n">
+      <c r="B22" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="C23" s="11">
-        <f>LbWk*Weeks*B23/DrumLb</f>
-        <v/>
-      </c>
-      <c r="D23" s="12">
-        <f>LbWk*Weeks*B23*(PCIlo-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="E23" s="12">
-        <f>LbWk*Weeks*B23*(PCImid-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="F23" s="12">
-        <f>LbWk*Weeks*B23*(PCIhi-SNPlb)</f>
-        <v/>
+      <c r="C22" s="14">
+        <f>LbWk*B22/DrumLb</f>
+        <v/>
+      </c>
+      <c r="D22" s="27">
+        <f>IF(C22&gt;=MinDrumsWk,"Yes",IF(B22&gt;=0.3,"Rounds up to the 1-drum minimum","NO — below supplier minimum"))</f>
+        <v/>
+      </c>
+      <c r="E22" s="15">
+        <f>IF(B22&gt;=0.3,LbWk*Weeks*MAX(B22,MinShare)*(PCImid-SNPlb),"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="28" t="inlineStr">
+        <is>
+          <t>This is why there is no 'low-cost insurance' version of Option A: the smallest second source anyone will sell us is one drum a week.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1616,7 +1674,7 @@
   <cols>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -1625,14 +1683,14 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>If SNP raises price on the volume it keeps (Year 1, PCI MID)</t>
+          <t>If SNP Inc. raises price on the volume it keeps (Year 1, PCI MID)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Losing a third of our volume may cost SNP its batch efficiency. A surcharge on the retained two-thirds compounds the premium.</t>
+          <t>Losing a third of our volume may cost SNP its batch efficiency. A surcharge on the retained ~2/3 compounds the premium.</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1707,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>SNP annual (2/3)</t>
+          <t>SNP annual (retained)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>PCI annual (1/3)</t>
+          <t>PCI annual</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -1669,126 +1727,126 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="21" t="n">
+      <c r="B6" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="21">
         <f>SNPlb*(1+B6)</f>
         <v/>
       </c>
-      <c r="D6" s="12">
-        <f>LbWk*Weeks*(1-Share)*C6</f>
-        <v/>
-      </c>
-      <c r="E6" s="12">
-        <f>LbWk*Weeks*Share*PCImid</f>
-        <v/>
-      </c>
-      <c r="F6" s="12">
+      <c r="D6" s="15">
+        <f>LbWk*Weeks*(1-EffShare)*C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="15">
+        <f>LbWk*Weeks*EffShare*PCImid</f>
+        <v/>
+      </c>
+      <c r="F6" s="15">
         <f>D6+E6</f>
         <v/>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="15">
         <f>F6-LbWk*Weeks*SNPlb</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="21" t="n">
+      <c r="B7" s="24" t="n">
         <v>0.05</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="21">
         <f>SNPlb*(1+B7)</f>
         <v/>
       </c>
-      <c r="D7" s="12">
-        <f>LbWk*Weeks*(1-Share)*C7</f>
-        <v/>
-      </c>
-      <c r="E7" s="12">
-        <f>LbWk*Weeks*Share*PCImid</f>
-        <v/>
-      </c>
-      <c r="F7" s="12">
+      <c r="D7" s="15">
+        <f>LbWk*Weeks*(1-EffShare)*C7</f>
+        <v/>
+      </c>
+      <c r="E7" s="15">
+        <f>LbWk*Weeks*EffShare*PCImid</f>
+        <v/>
+      </c>
+      <c r="F7" s="15">
         <f>D7+E7</f>
         <v/>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="15">
         <f>F7-LbWk*Weeks*SNPlb</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="21" t="n">
+      <c r="B8" s="24" t="n">
         <v>0.1</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="21">
         <f>SNPlb*(1+B8)</f>
         <v/>
       </c>
-      <c r="D8" s="12">
-        <f>LbWk*Weeks*(1-Share)*C8</f>
-        <v/>
-      </c>
-      <c r="E8" s="12">
-        <f>LbWk*Weeks*Share*PCImid</f>
-        <v/>
-      </c>
-      <c r="F8" s="12">
+      <c r="D8" s="15">
+        <f>LbWk*Weeks*(1-EffShare)*C8</f>
+        <v/>
+      </c>
+      <c r="E8" s="15">
+        <f>LbWk*Weeks*EffShare*PCImid</f>
+        <v/>
+      </c>
+      <c r="F8" s="15">
         <f>D8+E8</f>
         <v/>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="15">
         <f>F8-LbWk*Weeks*SNPlb</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="21" t="n">
+      <c r="B9" s="24" t="n">
         <v>0.2</v>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="21">
         <f>SNPlb*(1+B9)</f>
         <v/>
       </c>
-      <c r="D9" s="12">
-        <f>LbWk*Weeks*(1-Share)*C9</f>
-        <v/>
-      </c>
-      <c r="E9" s="12">
-        <f>LbWk*Weeks*Share*PCImid</f>
-        <v/>
-      </c>
-      <c r="F9" s="12">
+      <c r="D9" s="15">
+        <f>LbWk*Weeks*(1-EffShare)*C9</f>
+        <v/>
+      </c>
+      <c r="E9" s="15">
+        <f>LbWk*Weeks*EffShare*PCImid</f>
+        <v/>
+      </c>
+      <c r="F9" s="15">
         <f>D9+E9</f>
         <v/>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="15">
         <f>F9-LbWk*Weeks*SNPlb</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="21" t="n">
+      <c r="B10" s="24" t="n">
         <v>0.33</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="21">
         <f>SNPlb*(1+B10)</f>
         <v/>
       </c>
-      <c r="D10" s="12">
-        <f>LbWk*Weeks*(1-Share)*C10</f>
-        <v/>
-      </c>
-      <c r="E10" s="12">
-        <f>LbWk*Weeks*Share*PCImid</f>
-        <v/>
-      </c>
-      <c r="F10" s="12">
+      <c r="D10" s="15">
+        <f>LbWk*Weeks*(1-EffShare)*C10</f>
+        <v/>
+      </c>
+      <c r="E10" s="15">
+        <f>LbWk*Weeks*EffShare*PCImid</f>
+        <v/>
+      </c>
+      <c r="F10" s="15">
         <f>D10+E10</f>
         <v/>
       </c>
-      <c r="G10" s="12">
+      <c r="G10" s="15">
         <f>F10-LbWk*Weeks*SNPlb</f>
         <v/>
       </c>
@@ -1804,10 +1862,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G14"/>
+  <dimension ref="B2:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -1825,14 +1883,14 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>A second source is justified only if: annual premium &lt;= P(SNP disruption in a year) x loss the second source would AVOID. Note: at 1/3 share, 2/3 of volume is still exposed unless the second source can ramp.</t>
+          <t>Option A is justified only if: annual premium &lt;= P(SNP disruption in a year) x loss the second source would AVOID. ~2/3 of volume is still exposed until PCI can ramp.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Option</t>
+          <t>Option A price case</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1862,139 +1920,112 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>A — dual @ PCI LOW</t>
-        </is>
-      </c>
-      <c r="C6" s="12">
-        <f>LbWk*Weeks*Share*(PCIlo-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="D6" s="12">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>PCI LOW $2.50</t>
+        </is>
+      </c>
+      <c r="C6" s="15">
+        <f>LbWk*Weeks*EffShare*(PCIlo-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="D6" s="15">
         <f>C6/0.02</f>
         <v/>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="15">
         <f>C6/0.05</f>
         <v/>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="15">
         <f>C6/0.1</f>
         <v/>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="15">
         <f>C6/0.2</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>A — dual @ PCI MID</t>
-        </is>
-      </c>
-      <c r="C7" s="12">
-        <f>LbWk*Weeks*Share*(PCImid-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="D7" s="12">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>PCI MID $3.75</t>
+        </is>
+      </c>
+      <c r="C7" s="15">
+        <f>LbWk*Weeks*EffShare*(PCImid-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="D7" s="15">
         <f>C7/0.02</f>
         <v/>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="15">
         <f>C7/0.05</f>
         <v/>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="15">
         <f>C7/0.1</f>
         <v/>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="15">
         <f>C7/0.2</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>A — dual @ PCI HIGH</t>
-        </is>
-      </c>
-      <c r="C8" s="12">
-        <f>LbWk*Weeks*Share*(PCIhi-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="D8" s="12">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>PCI HIGH $5.00</t>
+        </is>
+      </c>
+      <c r="C8" s="15">
+        <f>LbWk*Weeks*EffShare*(PCIhi-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="D8" s="15">
         <f>C8/0.02</f>
         <v/>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="15">
         <f>C8/0.05</f>
         <v/>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="15">
         <f>C8/0.1</f>
         <v/>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="15">
         <f>C8/0.2</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>C — warm 5% @ PCI MID</t>
-        </is>
-      </c>
-      <c r="C9" s="12">
-        <f>LbWk*Weeks*WarmShare*(PCImid-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="D9" s="12">
-        <f>C9/0.02</f>
-        <v/>
-      </c>
-      <c r="E9" s="12">
-        <f>C9/0.05</f>
-        <v/>
-      </c>
-      <c r="F9" s="12">
-        <f>C9/0.1</f>
-        <v/>
-      </c>
-      <c r="G9" s="12">
-        <f>C9/0.2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Read: each cell = the avoided loss a disruption would have to cause for the premium to pay off. Compare to Inputs 'Cost of a 6-month SNP outage'.</t>
-        </is>
+    <row r="10">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Read: each cell = the avoided loss an SNP outage would have to cause for the premium to pay off. Compare to Inputs 'Cost of a 6-month SNP Inc. outage'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Expected annual loss with NO second source = Pdis x Dcost:</t>
+        </is>
+      </c>
+      <c r="D12" s="20">
+        <f>Pdis*Dcost</f>
+        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>Expected annual loss with NO second source = Pdis x Dcost:</t>
-        </is>
-      </c>
-      <c r="D13" s="17">
-        <f>Pdis*Dcost</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>Verdict @ PCI MID, 1/3 share:</t>
-        </is>
-      </c>
-      <c r="D14">
-        <f>IF(D13&gt;=C7,"Premium is justified","Premium exceeds expected loss")</f>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Verdict @ PCI MID:</t>
+        </is>
+      </c>
+      <c r="D13">
+        <f>IF(D12&gt;=C7,"Option A is justified","Premium exceeds expected loss — Option B")</f>
         <v/>
       </c>
     </row>
@@ -2009,19 +2040,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E13"/>
+  <dimension ref="B2:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>The three options, side by side (Year 1, PCI MID unless noted)</t>
+          <t>The two options, side by side (Year 1, PCI MID unless noted)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>There is no smaller version of A: the supplier minimum is one drum a week.</t>
         </is>
       </c>
     </row>
@@ -2029,184 +2066,143 @@
       <c r="B5" s="3" t="inlineStr"/>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>A — Dual-source now (1/3)</t>
+          <t>A — Second source (PCI Manufacturing) at ~1/3</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>B — Single + strengthen SNP</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>C — Warm backup (5%)</t>
+          <t>B — Single source (SNP Inc.) + strengthen</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Annual purchase cost</t>
         </is>
       </c>
-      <c r="C6" s="22">
-        <f>LbWk*Weeks*(1-Share)*SNPlb+LbWk*Weeks*Share*PCImid</f>
-        <v/>
-      </c>
-      <c r="D6" s="22">
+      <c r="C6" s="29">
+        <f>LbWk*Weeks*(1-EffShare)*SNPlb+LbWk*Weeks*EffShare*PCImid</f>
+        <v/>
+      </c>
+      <c r="D6" s="29">
         <f>LbWk*Weeks*SNPlb</f>
         <v/>
       </c>
-      <c r="E6" s="22">
-        <f>LbWk*Weeks*(1-WarmShare)*SNPlb+LbWk*Weeks*WarmShare*PCImid</f>
-        <v/>
-      </c>
     </row>
     <row r="7">
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Premium vs today</t>
         </is>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="29">
         <f>B6-LbWk*Weeks*SNPlb</f>
         <v/>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>0 (+ small continuity spend)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>One-time qualification</t>
+        </is>
+      </c>
+      <c r="C8" s="29">
+        <f>QualCost</f>
+        <v/>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>0 (plan/document only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>5-yr premium (10% growth)</t>
+        </is>
+      </c>
+      <c r="C9" s="29">
+        <f>'5-Year'!L11</f>
+        <v/>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E7" s="22">
-        <f>D6-LbWk*Weeks*SNPlb</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>One-time qualification</t>
-        </is>
-      </c>
-      <c r="C8" s="22">
-        <f>QualCost</f>
-        <v/>
-      </c>
-      <c r="D8" s="23" t="inlineStr">
-        <is>
-          <t>0 (plan/document only)</t>
-        </is>
-      </c>
-      <c r="E8" s="22">
-        <f>QualCost</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>5-yr premium (10% growth)</t>
-        </is>
-      </c>
-      <c r="C9" s="22">
-        <f>B7*(1+(1+Growth)+(1+Growth)^2+(1+Growth)^3+(1+Growth)^4)</f>
-        <v/>
-      </c>
-      <c r="D9" s="23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E9" s="22">
-        <f>D7*(1+(1+Growth)+(1+Growth)^2+(1+Growth)^3+(1+Growth)^4)</f>
-        <v/>
-      </c>
     </row>
     <row r="10">
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Volume still exposed if SNP fails</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>2/3 (until PCI ramps)</t>
-        </is>
-      </c>
-      <c r="D10" s="23" t="inlineStr">
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>~2/3 (until PCI ramps — unconfirmed)</t>
+        </is>
+      </c>
+      <c r="D10" s="30" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>95% (until PCI ramps)</t>
-        </is>
-      </c>
     </row>
     <row r="11">
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Time to recover if SNP fails</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C11" s="30" t="inlineStr">
         <is>
           <t>weeks (PCI ramp)</t>
         </is>
       </c>
-      <c r="D11" s="23" t="inlineStr">
-        <is>
-          <t>6-12 months (cold start)</t>
-        </is>
-      </c>
-      <c r="E11" s="23" t="inlineStr">
-        <is>
-          <t>weeks-months (re-activate)</t>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>6-12 months cold start; 3-4 with kit current</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>Signal to SNP</t>
-        </is>
-      </c>
-      <c r="C12" s="23" t="inlineStr">
-        <is>
-          <t>Lost a third of volume</t>
-        </is>
-      </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Signal to SNP Inc.</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>Lost a third of its volume</t>
+        </is>
+      </c>
+      <c r="D12" s="30" t="inlineStr">
         <is>
           <t>Deeper partnership</t>
         </is>
       </c>
-      <c r="E12" s="23" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
     </row>
     <row r="13">
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>Compliance posture</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
+      <c r="C13" s="30" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="D13" s="23" t="inlineStr">
-        <is>
-          <t>Defensible if documented</t>
-        </is>
-      </c>
-      <c r="E13" s="23" t="inlineStr">
-        <is>
-          <t>Strong</t>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>Defensible if risk + plan documented</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deck v4 + workbook: PCI real quote ($3.50/lb per 5-drum batch; $6 below)
- Workbook: new tabs Supplier Quotes, PCI Quote Scenarios (1/3 share, 5-yr,
  break-even, block-rotation logistics), PCI Experiment; Inputs gain PCIq/PCIsub/PCIbatch
- Charts: price per lb side by side; annual cost side by side
- Deck v4 (11 slides): detailed outline, what changed, two comparison slides,
  PCI experiment at what cost, 5-drum-batch logistics, strategy propositions
  A/B/B-plus, why decide now, recommendation & asks, appendix; notes on all

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
@@ -8,11 +8,14 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5-Year" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SNP Re-price" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Break-even" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Quotes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCI Quote Scenarios" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCI Experiment" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5-Year" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SNP Re-price" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Break-even" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="DrumLb">Inputs!$C$6</definedName>
@@ -34,6 +37,9 @@
     <definedName name="QualCost">Inputs!$C$22</definedName>
     <definedName name="Pdis">Inputs!$C$23</definedName>
     <definedName name="Dcost">Inputs!$C$24</definedName>
+    <definedName name="PCIq">Inputs!$C$27</definedName>
+    <definedName name="PCIsub">Inputs!$C$28</definedName>
+    <definedName name="PCIbatch">Inputs!$C$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -41,13 +47,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="167" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="169" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,8 +103,20 @@
       <color rgb="001F3864"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -128,6 +148,16 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -155,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -191,6 +221,48 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -558,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D24"/>
+  <dimension ref="B2:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="2" max="2"/>
@@ -880,12 +952,1253 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="B26" s="31" t="inlineStr">
+        <is>
+          <t>PCI MANUFACTURING — REAL QUOTE (2026-09-28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>PCI quoted price — one batch of 5 drums ($/lb)</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Real quote. CONFIRM: delivered? materials, drum, freight included? validity period?</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>PCI price — orders below one batch ($/lb)</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Real quote. Makes any sub-batch (e.g. 1 drum/week) uneconomic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>PCI batch size (drums)</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>One batch = 5 drums = 2,250 lb = ~12 days of full demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>The $2.50 / $3.75 / $5.00 rows above were the pre-quote forecast; keep for history. The quote ($3.50) sits at the forecast mid.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>All price points on the table — real quotes vs references</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>One place for every $/lb figure used anywhere in the analysis, with its basis. Real quotes in green; references in grey; superseded assumptions in amber.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>$/lb finished</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Basis / terms</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Date / reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>SNP Inc. (Durham, NC) — incumbent</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D6" s="34" t="inlineStr">
+        <is>
+          <t>Delivered, all-in. 1/450-lb drum. ~2.9 drums/week today.</t>
+        </is>
+      </c>
+      <c r="E6" s="34" t="inlineStr">
+        <is>
+          <t>REAL QUOTE</t>
+        </is>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>Active sole source</t>
+        </is>
+      </c>
+      <c r="G6" s="34" t="inlineStr">
+        <is>
+          <t>SNP Estimate 012726-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>PCI Manufacturing (St. Louis, MO) — one 5-drum batch</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D7" s="34" t="inlineStr">
+        <is>
+          <t>One batch = 5 drums (2,250 lb). Confirm delivered/all-in and validity.</t>
+        </is>
+      </c>
+      <c r="E7" s="34" t="inlineStr">
+        <is>
+          <t>REAL QUOTE</t>
+        </is>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>Capable — experiment successful; not yet contracted</t>
+        </is>
+      </c>
+      <c r="G7" s="34" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>PCI Manufacturing — below one batch</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" s="34" t="inlineStr">
+        <is>
+          <t>Any order smaller than 5 drums (e.g. 1 drum/week).</t>
+        </is>
+      </c>
+      <c r="E8" s="34" t="inlineStr">
+        <is>
+          <t>REAL QUOTE</t>
+        </is>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>Uneconomic version</t>
+        </is>
+      </c>
+      <c r="G8" s="34" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>CJB Applied Technologies (Valdosta, GA)</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>8.42</v>
+      </c>
+      <c r="D9" s="34" t="inlineStr">
+        <is>
+          <t>$8.00–8.50/lb toll EXCLUDING materials + ~$75/drum resin = ~$8.42 landed. Qual fee $4,900.</t>
+        </is>
+      </c>
+      <c r="E9" s="34" t="inlineStr">
+        <is>
+          <t>REAL QUOTE</t>
+        </is>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>Eliminated on price (~11x SNP)</t>
+        </is>
+      </c>
+      <c r="G9" s="34" t="inlineStr">
+        <is>
+          <t>CJB email 'RE: mix test'</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>Market reference — LOW</t>
+        </is>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D10" s="37" t="inlineStr">
+        <is>
+          <t>Resin floor + lean labor ($40/hr, 25% margin) + regional 1-drum freight</t>
+        </is>
+      </c>
+      <c r="E10" s="37" t="inlineStr">
+        <is>
+          <t>TRIANGULATED</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="inlineStr">
+        <is>
+          <t>Market Research tab (cost-scenarios workbook)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>Market reference — BASE</t>
+        </is>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D11" s="37" t="inlineStr">
+        <is>
+          <t>Same build-up at typical conversion</t>
+        </is>
+      </c>
+      <c r="E11" s="37" t="inlineStr">
+        <is>
+          <t>TRIANGULATED</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="G11" s="37" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>Market reference — HIGH</t>
+        </is>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="D12" s="37" t="inlineStr">
+        <is>
+          <t>Anchored by retail comp ~$2.03/lb bulk PVA solution + freight</t>
+        </is>
+      </c>
+      <c r="E12" s="37" t="inlineStr">
+        <is>
+          <t>TRIANGULATED</t>
+        </is>
+      </c>
+      <c r="F12" s="37" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="G12" s="37" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>Material floor</t>
+        </is>
+      </c>
+      <c r="C13" s="36" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D13" s="37" t="inlineStr">
+        <is>
+          <t>PVA resin $1.26–1.60/lb x 11% solids = $0.16–0.20</t>
+        </is>
+      </c>
+      <c r="E13" s="37" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F13" s="37" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="G13" s="37" t="inlineStr">
+        <is>
+          <t>ChemAnalyst / IMARC 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>July 2026 assumption (KPI deck)</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="n">
+        <v>1.125</v>
+      </c>
+      <c r="D14" s="40" t="inlineStr">
+        <is>
+          <t>'$1.00–1.25/lb, ~35% share, ~$6–12k/yr insurance'</t>
+        </is>
+      </c>
+      <c r="E14" s="40" t="inlineStr">
+        <is>
+          <t>ASSUMPTION</t>
+        </is>
+      </c>
+      <c r="F14" s="40" t="inlineStr">
+        <is>
+          <t>SUPERSEDED by PCI quote</t>
+        </is>
+      </c>
+      <c r="G14" s="40" t="inlineStr">
+        <is>
+          <t>KPI review deck 2026-07-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>Pre-quote forecast (this deck, Sept)</t>
+        </is>
+      </c>
+      <c r="C15" s="39" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D15" s="40" t="inlineStr">
+        <is>
+          <t>$2.50 low / $3.75 mid / $5.00 high</t>
+        </is>
+      </c>
+      <c r="E15" s="40" t="inlineStr">
+        <is>
+          <t>ASSUMPTION</t>
+        </is>
+      </c>
+      <c r="F15" s="40" t="inlineStr">
+        <is>
+          <t>SUPERSEDED by PCI quote (quote = mid)</t>
+        </is>
+      </c>
+      <c r="G15" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:I31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>What PCI's real quote means — Year 1 and five years</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Second source at one-third of demand = 50 drums/yr = 10 batches of 5. Formulas reference Inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Drums to PCI / yr</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>PCI $/lb</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>PCI annual $</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>SNP annual $ (retained)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Total $</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Premium vs all-SNP</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>x today's spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>All-SNP (today)</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="21">
+        <f>SNPlb</f>
+        <v/>
+      </c>
+      <c r="E6" s="15">
+        <f>C6*DrumLb*D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="15">
+        <f>(LbWk*Weeks-C6*DrumLb)*SNPlb</f>
+        <v/>
+      </c>
+      <c r="G6" s="15">
+        <f>E6+F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="15">
+        <f>G6-LbWk*Weeks*SNPlb</f>
+        <v/>
+      </c>
+      <c r="I6" s="41">
+        <f>H6/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="42" t="inlineStr">
+        <is>
+          <t>A — PCI at 1/3, 5-drum batches (10/yr)</t>
+        </is>
+      </c>
+      <c r="C7" s="43" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" s="44">
+        <f>PCIq</f>
+        <v/>
+      </c>
+      <c r="E7" s="45">
+        <f>C7*DrumLb*D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="45">
+        <f>(LbWk*Weeks-C7*DrumLb)*SNPlb</f>
+        <v/>
+      </c>
+      <c r="G7" s="45">
+        <f>E7+F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="45">
+        <f>G7-LbWk*Weeks*SNPlb</f>
+        <v/>
+      </c>
+      <c r="I7" s="46">
+        <f>H7/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>A — PCI 1 drum/week, below-batch price</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>52</v>
+      </c>
+      <c r="D8" s="21">
+        <f>PCIsub</f>
+        <v/>
+      </c>
+      <c r="E8" s="15">
+        <f>C8*DrumLb*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="15">
+        <f>(LbWk*Weeks-C8*DrumLb)*SNPlb</f>
+        <v/>
+      </c>
+      <c r="G8" s="15">
+        <f>E8+F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="15">
+        <f>G8-LbWk*Weeks*SNPlb</f>
+        <v/>
+      </c>
+      <c r="I8" s="41">
+        <f>H8/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>A — PCI at 1/3 but below-batch price (for reference)</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" s="21">
+        <f>PCIsub</f>
+        <v/>
+      </c>
+      <c r="E9" s="15">
+        <f>C9*DrumLb*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="15">
+        <f>(LbWk*Weeks-C9*DrumLb)*SNPlb</f>
+        <v/>
+      </c>
+      <c r="G9" s="15">
+        <f>E9+F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="15">
+        <f>G9-LbWk*Weeks*SNPlb</f>
+        <v/>
+      </c>
+      <c r="I9" s="41">
+        <f>H9/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>CJB at 1/3 (for scale)</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" s="21">
+        <f>CJBlb</f>
+        <v/>
+      </c>
+      <c r="E10" s="15">
+        <f>C10*DrumLb*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="15">
+        <f>(LbWk*Weeks-C10*DrumLb)*SNPlb</f>
+        <v/>
+      </c>
+      <c r="G10" s="15">
+        <f>E10+F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="15">
+        <f>G10-LbWk*Weeks*SNPlb</f>
+        <v/>
+      </c>
+      <c r="I10" s="41">
+        <f>H10/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="47" t="inlineStr">
+        <is>
+          <t>Five years at 1/3 share, PCI $3.50, volume +10%/yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Volume (lb)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Lb to PCI (1/3)</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Batches of 5 (rounded)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Premium ($2.75/lb x lb to PCI)</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Cumulative</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="12">
+        <f>LbWk*Weeks*(1+Growth)^(1-1)</f>
+        <v/>
+      </c>
+      <c r="D14" s="12">
+        <f>C14/3</f>
+        <v/>
+      </c>
+      <c r="E14" s="12">
+        <f>ROUND(D14/DrumLb/PCIbatch,0)</f>
+        <v/>
+      </c>
+      <c r="F14" s="15">
+        <f>D14*(PCIq-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="G14" s="15">
+        <f>F14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="12">
+        <f>LbWk*Weeks*(1+Growth)^(2-1)</f>
+        <v/>
+      </c>
+      <c r="D15" s="12">
+        <f>C15/3</f>
+        <v/>
+      </c>
+      <c r="E15" s="12">
+        <f>ROUND(D15/DrumLb/PCIbatch,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="15">
+        <f>D15*(PCIq-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="G15" s="15">
+        <f>G14+F15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="12">
+        <f>LbWk*Weeks*(1+Growth)^(3-1)</f>
+        <v/>
+      </c>
+      <c r="D16" s="12">
+        <f>C16/3</f>
+        <v/>
+      </c>
+      <c r="E16" s="12">
+        <f>ROUND(D16/DrumLb/PCIbatch,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="15">
+        <f>D16*(PCIq-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="G16" s="15">
+        <f>G15+F16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="12">
+        <f>LbWk*Weeks*(1+Growth)^(4-1)</f>
+        <v/>
+      </c>
+      <c r="D17" s="12">
+        <f>C17/3</f>
+        <v/>
+      </c>
+      <c r="E17" s="12">
+        <f>ROUND(D17/DrumLb/PCIbatch,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="15">
+        <f>D17*(PCIq-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="G17" s="15">
+        <f>G16+F17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" s="12">
+        <f>LbWk*Weeks*(1+Growth)^(5-1)</f>
+        <v/>
+      </c>
+      <c r="D18" s="12">
+        <f>C18/3</f>
+        <v/>
+      </c>
+      <c r="E18" s="12">
+        <f>ROUND(D18/DrumLb/PCIbatch,0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="15">
+        <f>D18*(PCIq-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="G18" s="15">
+        <f>G17+F18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="47" t="inlineStr">
+        <is>
+          <t>Break-even — outage cost that justifies the premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Premium (Y1)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>p = 2%</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>p = 5%</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>p = 10%</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>p = 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="15">
+        <f>H7</f>
+        <v/>
+      </c>
+      <c r="C22" s="15">
+        <f>B22/0.02</f>
+        <v/>
+      </c>
+      <c r="D22" s="15">
+        <f>B22/0.05</f>
+        <v/>
+      </c>
+      <c r="E22" s="15">
+        <f>B22/0.1</f>
+        <v/>
+      </c>
+      <c r="F22" s="15">
+        <f>B22/0.2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="47" t="inlineStr">
+        <is>
+          <t>Block-rotation logistics of a 5-drum batch (shelf life 18 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Batch size (lb)</t>
+        </is>
+      </c>
+      <c r="C25" s="12">
+        <f>PCIbatch*DrumLb</f>
+        <v/>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>Days of FULL demand in one batch</t>
+        </is>
+      </c>
+      <c r="C26" s="48">
+        <f>B25/(LbWk/7)</f>
+        <v/>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Must be consumed within the 18-day shelf life -&gt; use at full rate on receipt</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>Cycle length at 1/3 share (weeks)</t>
+        </is>
+      </c>
+      <c r="C27" s="48">
+        <f>B25/(LbWk/3)</f>
+        <v/>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>One PCI batch every ~5 weeks</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Weeks on SNP material per cycle</t>
+        </is>
+      </c>
+      <c r="C28" s="48">
+        <f>B27-B25/LbWk</f>
+        <v/>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>SNP sees a ~12-day gap every cycle: LUMPY demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>Days to consume a batch at 2/3 rate (needs 30-day shelf life)</t>
+        </is>
+      </c>
+      <c r="C29" s="48">
+        <f>B25/(LbWk*2/3/7)</f>
+        <v/>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>With a validated 30-day life, SNP can keep supplying at 1/3 rate during a PCI batch -&gt; smoother</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>One qualification batch — cost</t>
+        </is>
+      </c>
+      <c r="C30" s="15">
+        <f>B25*PCIq</f>
+        <v/>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>A single production-scale batch (Option B-plus)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>One qualification batch — premium over SNP</t>
+        </is>
+      </c>
+      <c r="C31" s="15">
+        <f>B25*(PCIq-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>~4% of annual volume; invisible to SNP's year</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="100" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>PCI Manufacturing — qualification experiment record</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>What was tested, what was found, what is still open. Source: email-chain summary 2026-09-22 + quote 2026-09-28.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Result / detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>Capability — 90–95 °C cook</t>
+        </is>
+      </c>
+      <c r="C6" s="34" t="inlineStr">
+        <is>
+          <t>PROVEN</t>
+        </is>
+      </c>
+      <c r="D6" s="34" t="inlineStr">
+        <is>
+          <t>Lab batches produced; dissolution achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>Viscosity (primary concern)</t>
+        </is>
+      </c>
+      <c r="C7" s="34" t="inlineStr">
+        <is>
+          <t>ROOT CAUSE FOUND</t>
+        </is>
+      </c>
+      <c r="D7" s="34" t="inlineStr">
+        <is>
+          <t>First sample 2,420 cP vs ~1,000 target; dilution to 10.8% solids -&gt; 1,590 cP; cause = elevated solids from water loss during processing; fix = water adjustment at end of mix</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>Agreed fresh-material spec</t>
+        </is>
+      </c>
+      <c r="C8" s="34" t="inlineStr">
+        <is>
+          <t>LOCKED</t>
+        </is>
+      </c>
+      <c r="D8" s="34" t="inlineStr">
+        <is>
+          <t>11% total solids; 900–1,100 cP fresh (Brookfield #3, 10 rpm, 25 °C); &lt;2,500 cP ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="B9" s="38" t="inlineStr">
+        <is>
+          <t>Colour</t>
+        </is>
+      </c>
+      <c r="C9" s="40" t="inlineStr">
+        <is>
+          <t>NOT A CRITERION</t>
+        </is>
+      </c>
+      <c r="D9" s="40" t="inlineStr">
+        <is>
+          <t>No formal spec; minor mismatch acceptable</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>Shelf-life study</t>
+        </is>
+      </c>
+      <c r="C10" s="40" t="inlineStr">
+        <is>
+          <t>REQUESTED</t>
+        </is>
+      </c>
+      <c r="D10" s="40" t="inlineStr">
+        <is>
+          <t>Viscosity every 3–5 days; trend to usable life (18 vs 30 days matters for batch logistics)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>Hydrogel compression strength</t>
+        </is>
+      </c>
+      <c r="C11" s="40" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="D11" s="40" t="inlineStr">
+        <is>
+          <t>vs current material — must hold on 100% PCI material under block rotation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>Cleaning / residual film</t>
+        </is>
+      </c>
+      <c r="C12" s="50" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D12" s="50" t="inlineStr">
+        <is>
+          <t>Film observed during processing; vinegar partially effective; procedure not final</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>Viscometer method basis</t>
+        </is>
+      </c>
+      <c r="C13" s="50" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D13" s="50" t="inlineStr">
+        <is>
+          <t>10 vs 60 rpm, LV vs RV series — all cP comparisons depend on it</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>Commercial — price</t>
+        </is>
+      </c>
+      <c r="C14" s="34" t="inlineStr">
+        <is>
+          <t>QUOTED</t>
+        </is>
+      </c>
+      <c r="D14" s="34" t="inlineStr">
+        <is>
+          <t>$3.50/lb at one 5-drum batch; $6.00/lb below a batch</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>Commercial — terms to confirm</t>
+        </is>
+      </c>
+      <c r="C15" s="50" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D15" s="50" t="inlineStr">
+        <is>
+          <t>Delivered/all-in? Validity? ~10 batches/yr on a ~5-week rhythm acceptable? Crisis ramp to ~3 batches/month? Resin grade/producer (sub-tier convergence with SNP)?</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="B16" s="38" t="inlineStr">
+        <is>
+          <t>What PCI has invested (unpaid)</t>
+        </is>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>NOTED</t>
+        </is>
+      </c>
+      <c r="D16" s="40" t="inlineStr">
+        <is>
+          <t>Two+ lab batches, dilution study, method work, revised process — months of engineering on a ~$50k/yr account</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1288,7 +2601,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1663,7 +2976,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1856,7 +3169,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2034,7 +3347,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Deck v4.2: remove the pre-quote 'What changed' slide; renumber outline, sections, cross-references and workbook Summary pointers
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
@@ -712,7 +712,7 @@
       </c>
       <c r="D6" s="52" t="inlineStr">
         <is>
-          <t>Slide 5 — identical in every bar</t>
+          <t>Slide 4 — identical in every bar</t>
         </is>
       </c>
     </row>
@@ -728,7 +728,7 @@
       </c>
       <c r="D7" s="52" t="inlineStr">
         <is>
-          <t>Slide 5</t>
+          <t>Slide 4</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       </c>
       <c r="D8" s="52" t="inlineStr">
         <is>
-          <t>Slide 5 — every option</t>
+          <t>Slide 4 — every option</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="D9" s="52" t="inlineStr">
         <is>
-          <t>Slides 3, 5, 7, 8</t>
+          <t>Slides 4, 6, 7</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D10" s="52" t="inlineStr">
         <is>
-          <t>Slide 5</t>
+          <t>Slide 4</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="D11" s="52" t="inlineStr">
         <is>
-          <t>Slide 5</t>
+          <t>Slide 4</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="D12" s="52" t="inlineStr">
         <is>
-          <t>Slides 5, 8</t>
+          <t>Slides 4, 7</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
       </c>
       <c r="D13" s="56" t="inlineStr">
         <is>
-          <t>Slides 5, 6, 8, 11</t>
+          <t>Slides 4, 5, 7, 10</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="D14" s="52" t="inlineStr">
         <is>
-          <t>Slide 5</t>
+          <t>Slide 4</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="D15" s="52" t="inlineStr">
         <is>
-          <t>Slide 5</t>
+          <t>Slide 4</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="D16" s="52" t="inlineStr">
         <is>
-          <t>Slide 5</t>
+          <t>Slide 4</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="D17" s="52" t="inlineStr">
         <is>
-          <t>Slides 6, 8</t>
+          <t>Slides 5, 7</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="D18" s="52" t="inlineStr">
         <is>
-          <t>Slide 11</t>
+          <t>Slide 10</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="D19" s="52" t="inlineStr">
         <is>
-          <t>Slide 11</t>
+          <t>Slide 10</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D21" s="52" t="inlineStr">
         <is>
-          <t>Slides 6, 8, 9, 11</t>
+          <t>Slides 5, 7, 8, 10</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="D22" s="52" t="inlineStr">
         <is>
-          <t>Slides 6, 9</t>
+          <t>Slides 5, 8</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="D23" s="52" t="inlineStr">
         <is>
-          <t>Slides 6, 8</t>
+          <t>Slides 5, 7</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="D24" s="52" t="inlineStr">
         <is>
-          <t>Slides 3, 7</t>
+          <t>Slide 6</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="D25" s="52" t="inlineStr">
         <is>
-          <t>Slide 7</t>
+          <t>Slide 6</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D26" s="52" t="inlineStr">
         <is>
-          <t>Slide 11</t>
+          <t>Slide 10</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="D27" s="52" t="inlineStr">
         <is>
-          <t>Slides 6, 8, 9, 11</t>
+          <t>Slides 5, 7, 8, 10</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="D28" s="52" t="inlineStr">
         <is>
-          <t>Slides 8, 9</t>
+          <t>Slides 7, 8</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="D29" s="52" t="inlineStr">
         <is>
-          <t>Slide 8</t>
+          <t>Slide 7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deck v4.3: remove the outline slide (outline is worked in conversation); slide-number references replaced by names
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
@@ -712,7 +712,7 @@
       </c>
       <c r="D6" s="52" t="inlineStr">
         <is>
-          <t>Slide 4 — identical in every bar</t>
+          <t>Annual-cost slide — identical in every bar</t>
         </is>
       </c>
     </row>
@@ -728,7 +728,7 @@
       </c>
       <c r="D7" s="52" t="inlineStr">
         <is>
-          <t>Slide 4</t>
+          <t>Annual-cost slide</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       </c>
       <c r="D8" s="52" t="inlineStr">
         <is>
-          <t>Slide 4 — every option</t>
+          <t>Annual-cost slide — every option</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="D9" s="52" t="inlineStr">
         <is>
-          <t>Slides 4, 6, 7</t>
+          <t>Annual-cost, logistics, options slides</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D10" s="52" t="inlineStr">
         <is>
-          <t>Slide 4</t>
+          <t>Annual-cost slide</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="D11" s="52" t="inlineStr">
         <is>
-          <t>Slide 4</t>
+          <t>Annual-cost slide</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="D12" s="52" t="inlineStr">
         <is>
-          <t>Slides 4, 7</t>
+          <t>Annual-cost and options slides</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
       </c>
       <c r="D13" s="56" t="inlineStr">
         <is>
-          <t>Slides 4, 5, 7, 10</t>
+          <t>Annual-cost, chronology, options, recommendation slides</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="D14" s="52" t="inlineStr">
         <is>
-          <t>Slide 4</t>
+          <t>Annual-cost slide</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="D15" s="52" t="inlineStr">
         <is>
-          <t>Slide 4</t>
+          <t>Annual-cost slide</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="D16" s="52" t="inlineStr">
         <is>
-          <t>Slide 4</t>
+          <t>Annual-cost slide</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="D17" s="52" t="inlineStr">
         <is>
-          <t>Slides 5, 7</t>
+          <t>Chronology and options slides</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="D18" s="52" t="inlineStr">
         <is>
-          <t>Slide 10</t>
+          <t>Recommendation slide</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="D19" s="52" t="inlineStr">
         <is>
-          <t>Slide 10</t>
+          <t>Recommendation slide</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D21" s="52" t="inlineStr">
         <is>
-          <t>Slides 5, 7, 8, 10</t>
+          <t>Chronology, options, keep-alive, recommendation slides</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="D22" s="52" t="inlineStr">
         <is>
-          <t>Slides 5, 8</t>
+          <t>Chronology and keep-alive slides</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="D23" s="52" t="inlineStr">
         <is>
-          <t>Slides 5, 7</t>
+          <t>Chronology and options slides</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="D24" s="52" t="inlineStr">
         <is>
-          <t>Slide 6</t>
+          <t>Logistics slide</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="D25" s="52" t="inlineStr">
         <is>
-          <t>Slide 6</t>
+          <t>Logistics slide</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D26" s="52" t="inlineStr">
         <is>
-          <t>Slide 10</t>
+          <t>Recommendation slide</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="D27" s="52" t="inlineStr">
         <is>
-          <t>Slides 5, 7, 8, 10</t>
+          <t>Chronology, options, keep-alive, recommendation slides</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="D28" s="52" t="inlineStr">
         <is>
-          <t>Slides 7, 8</t>
+          <t>Options and keep-alive slides</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="D29" s="52" t="inlineStr">
         <is>
-          <t>Slide 7</t>
+          <t>Options slide</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Annual-cost chart: Option 3 bars at 1/2/3 batches a year (blues); $6.00 bar as one drum a week (52 drums, ~1/3); reading-the-chart updated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
@@ -6106,7 +6106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I38"/>
+  <dimension ref="B2:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -6246,7 +6246,7 @@
     <row r="8">
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Option 1 — same 1/3 but ordered below batch size ($6.00) — chart bar</t>
+          <t>Option 1 — same 1/3 but ordered below batch size ($6.00) — reference</t>
         </is>
       </c>
       <c r="C8" s="12" t="n">
@@ -6382,14 +6382,14 @@
     <row r="12">
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Reference: 1 drum/week (52 drums) at the below-batch price</t>
+          <t>Option 3 — keep-alive: 3 batches (15 drums) / yr at $3.50</t>
         </is>
       </c>
       <c r="C12" s="12" t="n">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="D12" s="21">
-        <f>PCIsub</f>
+        <f>PCIq</f>
         <v/>
       </c>
       <c r="E12" s="15">
@@ -6413,76 +6413,85 @@
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="47" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>PCI $6.00 at 1 drum/week (52 drums, 23,400 lb ≈ 35% ≈ almost one-third) — chart bar</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>52</v>
+      </c>
+      <c r="D13" s="21">
+        <f>PCIsub</f>
+        <v/>
+      </c>
+      <c r="E13" s="15">
+        <f>C13*DrumLb*D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="15">
+        <f>(LbWk*Weeks-C13*DrumLb)*SNPlb</f>
+        <v/>
+      </c>
+      <c r="G13" s="15">
+        <f>E13+F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="15">
+        <f>G13-LbWk*Weeks*SNPlb</f>
+        <v/>
+      </c>
+      <c r="I13" s="41">
+        <f>H13/(LbWk*Weeks*SNPlb)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="47" t="inlineStr">
         <is>
           <t>Five years at 1/3 share (Option 1), PCI $3.50, volume +10%/yr</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="B15" s="3" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Volume (lb)</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Lb to PCI (1/3)</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Batches of 5 (rounded)</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Premium ($2.75/lb x lb to PCI)</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Cumulative</t>
         </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" s="12">
-        <f>LbWk*Weeks*(1+Growth)^(1-1)</f>
-        <v/>
-      </c>
-      <c r="D16" s="12">
-        <f>C16/3</f>
-        <v/>
-      </c>
-      <c r="E16" s="12">
-        <f>ROUND(D16/DrumLb/PCIbatch,0)</f>
-        <v/>
-      </c>
-      <c r="F16" s="15">
-        <f>D16*(PCIq-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="G16" s="15">
-        <f>F16</f>
-        <v/>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" s="12">
-        <f>LbWk*Weeks*(1+Growth)^(2-1)</f>
+        <f>LbWk*Weeks*(1+Growth)^(1-1)</f>
         <v/>
       </c>
       <c r="D17" s="12">
@@ -6498,16 +6507,16 @@
         <v/>
       </c>
       <c r="G17" s="15">
-        <f>G16+F17</f>
+        <f>F17</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C18" s="12">
-        <f>LbWk*Weeks*(1+Growth)^(3-1)</f>
+        <f>LbWk*Weeks*(1+Growth)^(2-1)</f>
         <v/>
       </c>
       <c r="D18" s="12">
@@ -6529,10 +6538,10 @@
     </row>
     <row r="19">
       <c r="B19" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19" s="12">
-        <f>LbWk*Weeks*(1+Growth)^(4-1)</f>
+        <f>LbWk*Weeks*(1+Growth)^(3-1)</f>
         <v/>
       </c>
       <c r="D19" s="12">
@@ -6554,10 +6563,10 @@
     </row>
     <row r="20">
       <c r="B20" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C20" s="12">
-        <f>LbWk*Weeks*(1+Growth)^(5-1)</f>
+        <f>LbWk*Weeks*(1+Growth)^(4-1)</f>
         <v/>
       </c>
       <c r="D20" s="12">
@@ -6577,247 +6586,272 @@
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="47" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" s="12">
+        <f>LbWk*Weeks*(1+Growth)^(5-1)</f>
+        <v/>
+      </c>
+      <c r="D21" s="12">
+        <f>C21/3</f>
+        <v/>
+      </c>
+      <c r="E21" s="12">
+        <f>ROUND(D21/DrumLb/PCIbatch,0)</f>
+        <v/>
+      </c>
+      <c r="F21" s="15">
+        <f>D21*(PCIq-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="G21" s="15">
+        <f>G20+F21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="47" t="inlineStr">
         <is>
           <t>Break-even — outage cost that justifies the premium</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="B23" s="3" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Premium (Y1)</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>p = 2%</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>p = 5%</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>p = 10%</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>p = 20%</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="15">
+    <row r="25">
+      <c r="B25" s="15">
         <f>H7</f>
         <v/>
       </c>
-      <c r="C24" s="15">
-        <f>B24/0.02</f>
-        <v/>
-      </c>
-      <c r="D24" s="15">
-        <f>B24/0.05</f>
-        <v/>
-      </c>
-      <c r="E24" s="15">
-        <f>B24/0.1</f>
-        <v/>
-      </c>
-      <c r="F24" s="15">
-        <f>B24/0.2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="47" t="inlineStr">
+      <c r="C25" s="15">
+        <f>B25/0.02</f>
+        <v/>
+      </c>
+      <c r="D25" s="15">
+        <f>B25/0.05</f>
+        <v/>
+      </c>
+      <c r="E25" s="15">
+        <f>B25/0.1</f>
+        <v/>
+      </c>
+      <c r="F25" s="15">
+        <f>B25/0.2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="47" t="inlineStr">
         <is>
           <t>Block-rotation logistics of a 5-drum batch (shelf life 18 days)</t>
         </is>
       </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>Batch size (lb)</t>
-        </is>
-      </c>
-      <c r="C27" s="12">
-        <f>PCIbatch*DrumLb</f>
-        <v/>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>Days of FULL demand in one batch</t>
-        </is>
-      </c>
-      <c r="C28" s="48">
-        <f>B27/(LbWk/7)</f>
-        <v/>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>12.1 days — must be consumed within the shelf life -&gt; use at full rate on receipt</t>
-        </is>
-      </c>
+          <t>Batch size (lb)</t>
+        </is>
+      </c>
+      <c r="C28" s="12">
+        <f>PCIbatch*DrumLb</f>
+        <v/>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>Cycle length at 1/3 share (weeks)</t>
+          <t>Days of FULL demand in one batch</t>
         </is>
       </c>
       <c r="C29" s="48">
-        <f>B27/(LbWk/3)</f>
+        <f>B28/(LbWk/7)</f>
         <v/>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>One PCI batch every ~5 weeks (Year 1: 10 batches; ~15 by Year 5)</t>
+          <t>12.1 days — must be consumed within the shelf life -&gt; use at full rate on receipt</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>Weeks on SNP material per cycle</t>
+          <t>Cycle length at 1/3 share (weeks)</t>
         </is>
       </c>
       <c r="C30" s="48">
-        <f>B29-B27/LbWk</f>
+        <f>B28/(LbWk/3)</f>
         <v/>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Cadence is a choice: (i) block rotation = a ~12-day pause in SNP orders per cycle; (ii) SNP keeps ~2 drums/wk and we hold ~3 drums of rolling stock (peak ~8 drums, strict first-in-first-out) — the shelf-life study decides</t>
+          <t>One PCI batch every ~5 weeks (Year 1: 10 batches; ~15 by Year 5)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>Age of PCI drums on receipt (days: cook, release, transit) — INPUT</t>
-        </is>
-      </c>
-      <c r="C31" s="63" t="n">
-        <v>4</v>
+          <t>Weeks on SNP material per cycle</t>
+        </is>
+      </c>
+      <c r="C31" s="48">
+        <f>B30-B28/LbWk</f>
+        <v/>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Assumption: the 18-day clock starts at manufacture. Confirm PCI lead time and transit St. Louis -&gt; site</t>
+          <t>Cadence is a choice: (i) block rotation = a ~12-day pause in SNP orders per cycle; (ii) SNP keeps ~2 drums/wk and we hold ~3 drums of rolling stock (peak ~8 drums, strict first-in-first-out) — the shelf-life study decides</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>Usable days on receipt (18-day life)</t>
-        </is>
-      </c>
-      <c r="C32" s="48">
-        <f>18-B31</f>
-        <v/>
-      </c>
-      <c r="D32" s="2" t="inlineStr"/>
+          <t>Age of PCI drums on receipt (days: cook, release, transit) — INPUT</t>
+        </is>
+      </c>
+      <c r="C32" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Assumption: the 18-day clock starts at manufacture. Confirm PCI lead time and transit St. Louis -&gt; site</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>Slack in block rotation (days)</t>
+          <t>Usable days on receipt (18-day life)</t>
         </is>
       </c>
       <c r="C33" s="48">
-        <f>B32-B28</f>
-        <v/>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>~1–2 days: block rotation has almost no margin at 18 days; a validated 21-day life gives real margin</t>
-        </is>
-      </c>
+        <f>18-B32</f>
+        <v/>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="B34" s="17" t="inlineStr">
         <is>
-          <t>Days to consume a batch at 2/3 rate</t>
+          <t>Slack in block rotation (days)</t>
         </is>
       </c>
       <c r="C34" s="48">
-        <f>B27/(LbWk*2/3/7)</f>
+        <f>B33-B29</f>
         <v/>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>18.2 days — needs a validated life longer than 18.2 days plus the age on receipt</t>
+          <t>~1–2 days: block rotation has almost no margin at 18 days; a validated 21-day life gives real margin</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="17" t="inlineStr">
         <is>
-          <t>Days to consume a batch at an exact 1/3 rate</t>
+          <t>Days to consume a batch at 2/3 rate</t>
         </is>
       </c>
       <c r="C35" s="48">
-        <f>B27/(LbWk/3/7)</f>
+        <f>B28/(LbWk*2/3/7)</f>
         <v/>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>36.3 days — a true one-third blend needs a ~40-day validated life</t>
+          <t>18.2 days — needs a validated life longer than 18.2 days plus the age on receipt</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="17" t="inlineStr">
         <is>
-          <t>Minimum PCI share of rate under a 30-day life</t>
-        </is>
-      </c>
-      <c r="C36" s="24">
-        <f>B27/((30-B31)*LbWk/7)</f>
+          <t>Days to consume a batch at an exact 1/3 rate</t>
+        </is>
+      </c>
+      <c r="C36" s="48">
+        <f>B28/(LbWk/3/7)</f>
         <v/>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>~47% at 4 days' age: even a 30-day life does not allow a one-third blend</t>
+          <t>36.3 days — a true one-third blend needs a ~40-day validated life</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="17" t="inlineStr">
         <is>
-          <t>One qualification batch — cost</t>
-        </is>
-      </c>
-      <c r="C37" s="15">
-        <f>B27*PCIq</f>
+          <t>Minimum PCI share of rate under a 30-day life</t>
+        </is>
+      </c>
+      <c r="C37" s="24">
+        <f>B28/((30-B32)*LbWk/7)</f>
         <v/>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>A single production-scale batch (Option B-plus); $7.9k gross</t>
+          <t>~47% at 4 days' age: even a 30-day life does not allow a one-third blend</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="17" t="inlineStr">
         <is>
+          <t>One qualification batch — cost</t>
+        </is>
+      </c>
+      <c r="C38" s="15">
+        <f>B28*PCIq</f>
+        <v/>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>A single production-scale batch (Option B-plus); $7.9k gross</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="17" t="inlineStr">
+        <is>
           <t>One qualification batch — premium over SNP</t>
         </is>
       </c>
-      <c r="C38" s="15">
-        <f>B27*(PCIq-SNPlb)</f>
-        <v/>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="C39" s="15">
+        <f>B28*(PCIq-SNPlb)</f>
+        <v/>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>3.3% of annual volume (2,250 of 67,600 lb); one ~12-day pause in SNP orders</t>
         </is>

</xml_diff>

<commit_message>
Chronology corrections: ArroChem and Columbus right kind of company but no heating capacity; APV estimated >= $3/lb (unconfirmed); 22 Sep = test results, not a root-cause finding
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
@@ -1842,7 +1842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G18"/>
+  <dimension ref="B2:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="2" max="2"/>
@@ -2022,77 +2022,77 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
+          <t>APV Engineered Coatings (Akron, OH) — no quote</t>
+        </is>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="37" t="inlineStr">
+        <is>
+          <t>On our call they considered $1.50/lb too cheap for our volume; we estimate at least $3.00/lb — NEVER CONFIRMED. Heat capability confirmed.</t>
+        </is>
+      </c>
+      <c r="E10" s="37" t="inlineStr">
+        <is>
+          <t>ESTIMATE</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>No quote received; reserve</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="inlineStr">
+        <is>
+          <t>APV call (2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="35" t="inlineStr">
+        <is>
           <t>Brenntag (distributor) — trial blends, Nov 2025 onward</t>
         </is>
       </c>
-      <c r="C10" s="36" t="inlineStr">
+      <c r="C11" s="36" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="D10" s="37" t="inlineStr">
+      <c r="D11" s="37" t="inlineStr">
         <is>
           <t>Tried our formula (125 grade and the requested grade): viscosity above range, unreadable on their viscometer. They stalled; no quote was ever received. Mar 2026: sent us a 125-grade resin sample instead.</t>
         </is>
       </c>
-      <c r="E10" s="37" t="inlineStr">
+      <c r="E11" s="37" t="inlineStr">
         <is>
           <t>NO QUOTE</t>
         </is>
       </c>
-      <c r="F10" s="37" t="inlineStr">
+      <c r="F11" s="37" t="inlineStr">
         <is>
           <t>Never met viscosity; no quote</t>
         </is>
       </c>
-      <c r="G10" s="37" t="inlineStr">
+      <c r="G11" s="37" t="inlineStr">
         <is>
           <t>Sam (Brenntag) emails</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="60" t="inlineStr">
-        <is>
-          <t>Market — COMPETITIVE quantity (drum scale, 30–55 gal)</t>
-        </is>
-      </c>
-      <c r="C11" s="61" t="n">
-        <v>2.32</v>
-      </c>
-      <c r="D11" s="62" t="inlineStr">
-        <is>
-          <t>Inferred from comparable pre-mixed PVA solutions sold today; range 2.20-5.03; n=7</t>
-        </is>
-      </c>
-      <c r="E11" s="62" t="inlineStr">
-        <is>
-          <t>MARKET STUDY</t>
-        </is>
-      </c>
-      <c r="F11" s="62" t="inlineStr">
-        <is>
-          <t>Reference — see Market Study tab</t>
-        </is>
-      </c>
-      <c r="G11" s="62" t="inlineStr">
-        <is>
-          <t>Verified market study 2026-09-28</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="60" t="inlineStr">
         <is>
-          <t>Market — LOW quantity (pints to 5-gal pails)</t>
+          <t>Market — COMPETITIVE quantity (drum scale, 30–55 gal)</t>
         </is>
       </c>
       <c r="C12" s="61" t="n">
-        <v>4.55</v>
+        <v>2.32</v>
       </c>
       <c r="D12" s="62" t="inlineStr">
         <is>
-          <t>Retail/lab packs; range 3.19-5.87; n=32</t>
+          <t>Inferred from comparable pre-mixed PVA solutions sold today; range 2.20-5.03; n=7</t>
         </is>
       </c>
       <c r="E12" s="62" t="inlineStr">
@@ -2114,160 +2114,190 @@
     <row r="13">
       <c r="B13" s="60" t="inlineStr">
         <is>
+          <t>Market — LOW quantity (pints to 5-gal pails)</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="D13" s="62" t="inlineStr">
+        <is>
+          <t>Retail/lab packs; range 3.19-5.87; n=32</t>
+        </is>
+      </c>
+      <c r="E13" s="62" t="inlineStr">
+        <is>
+          <t>MARKET STUDY</t>
+        </is>
+      </c>
+      <c r="F13" s="62" t="inlineStr">
+        <is>
+          <t>Reference — see Market Study tab</t>
+        </is>
+      </c>
+      <c r="G13" s="62" t="inlineStr">
+        <is>
+          <t>Verified market study 2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="60" t="inlineStr">
+        <is>
           <t>Market — HIGH quantity (totes / bulk / tonnage)</t>
         </is>
       </c>
-      <c r="C13" s="61" t="n">
+      <c r="C14" s="61" t="n">
         <v>1.01</v>
       </c>
-      <c r="D13" s="62" t="inlineStr">
+      <c r="D14" s="62" t="inlineStr">
         <is>
           <t>Bulk and contract pricing; range 0.28-1.04; n=5. Quality/regulatory context differs.</t>
         </is>
       </c>
-      <c r="E13" s="62" t="inlineStr">
+      <c r="E14" s="62" t="inlineStr">
         <is>
           <t>MARKET STUDY</t>
         </is>
       </c>
-      <c r="F13" s="62" t="inlineStr">
+      <c r="F14" s="62" t="inlineStr">
         <is>
           <t>Reference — see Market Study tab</t>
         </is>
       </c>
-      <c r="G13" s="62" t="inlineStr">
+      <c r="G14" s="62" t="inlineStr">
         <is>
           <t>Verified market study 2026-09-28</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="35" t="inlineStr">
-        <is>
-          <t>— Superseded / historical references (kept for the record) —</t>
-        </is>
-      </c>
-      <c r="C14" s="36" t="inlineStr"/>
-      <c r="D14" s="37" t="inlineStr"/>
-      <c r="E14" s="37" t="inlineStr"/>
-      <c r="F14" s="37" t="inlineStr"/>
-      <c r="G14" s="37" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>Triangulated market LOW / BASE / HIGH (Sept)</t>
-        </is>
-      </c>
-      <c r="C15" s="36" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="D15" s="37" t="inlineStr">
-        <is>
-          <t>$0.85 / $1.40 / $2.55 — resin floor + labor build-up + retail ceiling</t>
-        </is>
-      </c>
-      <c r="E15" s="37" t="inlineStr">
-        <is>
-          <t>TRIANGULATED</t>
-        </is>
-      </c>
-      <c r="F15" s="37" t="inlineStr">
-        <is>
-          <t>SUPERSEDED by market study</t>
-        </is>
-      </c>
-      <c r="G15" s="37" t="inlineStr">
-        <is>
-          <t>Market Research tab (cost-scenarios workbook)</t>
-        </is>
-      </c>
+          <t>— Superseded / historical references (kept for the record) —</t>
+        </is>
+      </c>
+      <c r="C15" s="36" t="inlineStr"/>
+      <c r="D15" s="37" t="inlineStr"/>
+      <c r="E15" s="37" t="inlineStr"/>
+      <c r="F15" s="37" t="inlineStr"/>
+      <c r="G15" s="37" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="B16" s="35" t="inlineStr">
         <is>
+          <t>Triangulated market LOW / BASE / HIGH (Sept)</t>
+        </is>
+      </c>
+      <c r="C16" s="36" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D16" s="37" t="inlineStr">
+        <is>
+          <t>$0.85 / $1.40 / $2.55 — resin floor + labor build-up + retail ceiling</t>
+        </is>
+      </c>
+      <c r="E16" s="37" t="inlineStr">
+        <is>
+          <t>TRIANGULATED</t>
+        </is>
+      </c>
+      <c r="F16" s="37" t="inlineStr">
+        <is>
+          <t>SUPERSEDED by market study</t>
+        </is>
+      </c>
+      <c r="G16" s="37" t="inlineStr">
+        <is>
+          <t>Market Research tab (cost-scenarios workbook)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="35" t="inlineStr">
+        <is>
           <t>Material floor</t>
         </is>
       </c>
-      <c r="C16" s="36" t="n">
+      <c r="C17" s="36" t="n">
         <v>0.18</v>
       </c>
-      <c r="D16" s="37" t="inlineStr">
+      <c r="D17" s="37" t="inlineStr">
         <is>
           <t>PVA resin $1.26–1.60/lb x 11% solids = $0.14–0.18 (upper bound plotted)</t>
         </is>
       </c>
-      <c r="E16" s="37" t="inlineStr">
+      <c r="E17" s="37" t="inlineStr">
         <is>
           <t>DERIVED</t>
         </is>
       </c>
-      <c r="F16" s="37" t="inlineStr">
+      <c r="F17" s="37" t="inlineStr">
         <is>
           <t>Reference only</t>
         </is>
       </c>
-      <c r="G16" s="37" t="inlineStr">
+      <c r="G17" s="37" t="inlineStr">
         <is>
           <t>ChemAnalyst / IMARC 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="38" t="inlineStr">
-        <is>
-          <t>July 2026 assumption (key performance indicator (KPI) review deck)</t>
-        </is>
-      </c>
-      <c r="C17" s="39" t="n">
-        <v>1.125</v>
-      </c>
-      <c r="D17" s="40" t="inlineStr">
-        <is>
-          <t>'$1.00–1.25/lb, ~35% share, ~$6–12k/yr insurance'</t>
-        </is>
-      </c>
-      <c r="E17" s="40" t="inlineStr">
-        <is>
-          <t>ASSUMPTION</t>
-        </is>
-      </c>
-      <c r="F17" s="40" t="inlineStr">
-        <is>
-          <t>SUPERSEDED by PCI quote</t>
-        </is>
-      </c>
-      <c r="G17" s="40" t="inlineStr">
-        <is>
-          <t>KPI review deck 2026-07-09</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="38" t="inlineStr">
         <is>
+          <t>July 2026 assumption (key performance indicator (KPI) review deck)</t>
+        </is>
+      </c>
+      <c r="C18" s="39" t="n">
+        <v>1.125</v>
+      </c>
+      <c r="D18" s="40" t="inlineStr">
+        <is>
+          <t>'$1.00–1.25/lb, ~35% share, ~$6–12k/yr insurance'</t>
+        </is>
+      </c>
+      <c r="E18" s="40" t="inlineStr">
+        <is>
+          <t>ASSUMPTION</t>
+        </is>
+      </c>
+      <c r="F18" s="40" t="inlineStr">
+        <is>
+          <t>SUPERSEDED by PCI quote</t>
+        </is>
+      </c>
+      <c r="G18" s="40" t="inlineStr">
+        <is>
+          <t>KPI review deck 2026-07-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="38" t="inlineStr">
+        <is>
           <t>Pre-quote forecast (this deck, Sept)</t>
         </is>
       </c>
-      <c r="C18" s="39" t="n">
+      <c r="C19" s="39" t="n">
         <v>3.75</v>
       </c>
-      <c r="D18" s="40" t="inlineStr">
+      <c r="D19" s="40" t="inlineStr">
         <is>
           <t>$2.50 low / $3.75 mid / $5.00 high</t>
         </is>
       </c>
-      <c r="E18" s="40" t="inlineStr">
+      <c r="E19" s="40" t="inlineStr">
         <is>
           <t>ASSUMPTION</t>
         </is>
       </c>
-      <c r="F18" s="40" t="inlineStr">
+      <c r="F19" s="40" t="inlineStr">
         <is>
           <t>SUPERSEDED by PCI quote (quote = mid)</t>
         </is>
       </c>
-      <c r="G18" s="40" t="inlineStr">
+      <c r="G19" s="40" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
@@ -6932,12 +6962,12 @@
       </c>
       <c r="C7" s="34" t="inlineStr">
         <is>
-          <t>ROOT CAUSE FOUND</t>
+          <t>ADJUSTED IN TEST</t>
         </is>
       </c>
       <c r="D7" s="34" t="inlineStr">
         <is>
-          <t>First sample 2,420 cP vs ~1,000 target; dilution to 10.8% solids -&gt; 1,590 cP; cause = elevated solids from water loss during processing; fix = water adjustment at end of mix</t>
+          <t>First sample 2,420 cP vs ~1,000 target; dilution to 10.8% solids -&gt; 1,590 cP; brought on target within the test by adjusting solids/water at end of mix (part of the test, not a separate root-cause finding)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbook: Price Curve tab (trend, band, values at each lot size); chronology file count corrected
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
@@ -11,13 +11,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Quotes" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Study" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCI Quote Scenarios" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCI Experiment" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5-Year" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SNP Re-price" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Break-even" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price Curve" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCI Quote Scenarios" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCI Experiment" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5-Year" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SNP Re-price" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Break-even" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="DrumLb">Inputs!$C$6</definedName>
@@ -49,13 +50,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="167" formatCode="0.0&quot;x&quot;"/>
     <numFmt numFmtId="168" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="170" formatCode="0.000"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -187,7 +189,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -296,6 +298,11 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1095,6 +1102,199 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>If SNP Inc. raises price on the volume it keeps (Year 1, PCI quote $3.50, 50 drums to PCI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Losing a third of our volume may cost SNP its batch efficiency. A surcharge on the retained ~2/3 compounds the premium.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>SNP surcharge</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>SNP $/lb</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>SNP annual (retained)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>PCI annual</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Premium vs today</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="21">
+        <f>SNPlb*(1+B6)</f>
+        <v/>
+      </c>
+      <c r="D6" s="15">
+        <f>LbWk*Weeks*(1-EffShare)*C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="15">
+        <f>LbWk*Weeks*EffShare*PCImid</f>
+        <v/>
+      </c>
+      <c r="F6" s="15">
+        <f>D6+E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="15">
+        <f>F6-LbWk*Weeks*SNPlb</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C7" s="21">
+        <f>SNPlb*(1+B7)</f>
+        <v/>
+      </c>
+      <c r="D7" s="15">
+        <f>LbWk*Weeks*(1-EffShare)*C7</f>
+        <v/>
+      </c>
+      <c r="E7" s="15">
+        <f>LbWk*Weeks*EffShare*PCImid</f>
+        <v/>
+      </c>
+      <c r="F7" s="15">
+        <f>D7+E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="15">
+        <f>F7-LbWk*Weeks*SNPlb</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="24" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C8" s="21">
+        <f>SNPlb*(1+B8)</f>
+        <v/>
+      </c>
+      <c r="D8" s="15">
+        <f>LbWk*Weeks*(1-EffShare)*C8</f>
+        <v/>
+      </c>
+      <c r="E8" s="15">
+        <f>LbWk*Weeks*EffShare*PCImid</f>
+        <v/>
+      </c>
+      <c r="F8" s="15">
+        <f>D8+E8</f>
+        <v/>
+      </c>
+      <c r="G8" s="15">
+        <f>F8-LbWk*Weeks*SNPlb</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="24" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C9" s="21">
+        <f>SNPlb*(1+B9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="15">
+        <f>LbWk*Weeks*(1-EffShare)*C9</f>
+        <v/>
+      </c>
+      <c r="E9" s="15">
+        <f>LbWk*Weeks*EffShare*PCImid</f>
+        <v/>
+      </c>
+      <c r="F9" s="15">
+        <f>D9+E9</f>
+        <v/>
+      </c>
+      <c r="G9" s="15">
+        <f>F9-LbWk*Weeks*SNPlb</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="24" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="C10" s="21">
+        <f>SNPlb*(1+B10)</f>
+        <v/>
+      </c>
+      <c r="D10" s="15">
+        <f>LbWk*Weeks*(1-EffShare)*C10</f>
+        <v/>
+      </c>
+      <c r="E10" s="15">
+        <f>LbWk*Weeks*EffShare*PCImid</f>
+        <v/>
+      </c>
+      <c r="F10" s="15">
+        <f>D10+E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="15">
+        <f>F10-LbWk*Weeks*SNPlb</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1267,7 +1467,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6136,6 +6336,310 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Price per lb vs. quantity per order — market trend, band and where each supplier sits</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Fit: log-log regression of verified market points (US packs 2 lb–20 gal, ≤$12/lb, plus ton-scale offers at 2,205 lb). Band = 10th–90th percentile of points around the trend; beyond 20 gal the top follows vendors' volume ladders flattening (~8%/doubling from $2.32 at 20 gal); floor = SNP's $0.75 (no US-delivered lot seen cheaper).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Trend coefficient A ($/lb at 1 lb)</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>8.301220449729895</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Trend exponent b</t>
+        </is>
+      </c>
+      <c r="C6" s="68" t="n">
+        <v>-0.2949856235683102</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Price change per doubling of lot</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>-0.1849195453748944</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Band: 10th-percentile ratio to trend</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>0.603671955514413</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Band: 90th-percentile ratio to trend</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>1.711030467025052</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Points used in fit</t>
+        </is>
+      </c>
+      <c r="C10" s="69" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="70" t="inlineStr">
+        <is>
+          <t>Quantity per order</t>
+        </is>
+      </c>
+      <c r="C12" s="70" t="inlineStr">
+        <is>
+          <t>lb</t>
+        </is>
+      </c>
+      <c r="D12" s="70" t="inlineStr">
+        <is>
+          <t>Trend $/lb</t>
+        </is>
+      </c>
+      <c r="E12" s="70" t="inlineStr">
+        <is>
+          <t>Band low $/lb</t>
+        </is>
+      </c>
+      <c r="F12" s="70" t="inlineStr">
+        <is>
+          <t>Band high $/lb</t>
+        </is>
+      </c>
+      <c r="G12" s="70" t="inlineStr">
+        <is>
+          <t>Real quote / point</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>1 gal</t>
+        </is>
+      </c>
+      <c r="C13" s="51" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D13" s="67" t="n">
+        <v>4.415467839760789</v>
+      </c>
+      <c r="E13" s="67" t="n">
+        <v>2.665494105339397</v>
+      </c>
+      <c r="F13" s="67" t="n">
+        <v>7.555</v>
+      </c>
+      <c r="G13" s="52" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>5 gal</t>
+        </is>
+      </c>
+      <c r="C14" s="51" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="D14" s="67" t="n">
+        <v>2.746569691723967</v>
+      </c>
+      <c r="E14" s="67" t="n">
+        <v>1.658027096759626</v>
+      </c>
+      <c r="F14" s="67" t="n">
+        <v>4.699464422347312</v>
+      </c>
+      <c r="G14" s="52" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>20 gal (largest US lot)</t>
+        </is>
+      </c>
+      <c r="C15" s="51" t="n">
+        <v>170</v>
+      </c>
+      <c r="D15" s="67" t="n">
+        <v>1.824700459266596</v>
+      </c>
+      <c r="E15" s="67" t="n">
+        <v>1.101520494473514</v>
+      </c>
+      <c r="F15" s="67" t="n">
+        <v>3.12211807899975</v>
+      </c>
+      <c r="G15" s="52" t="inlineStr">
+        <is>
+          <t>$2.32 US Composites</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>1 drum</t>
+        </is>
+      </c>
+      <c r="C16" s="51" t="n">
+        <v>450</v>
+      </c>
+      <c r="D16" s="67" t="n">
+        <v>1.369248895991172</v>
+      </c>
+      <c r="E16" s="67" t="n">
+        <v>0.826577158628942</v>
+      </c>
+      <c r="F16" s="67" t="n">
+        <v>3.530934857171929</v>
+      </c>
+      <c r="G16" s="52" t="inlineStr">
+        <is>
+          <t>PCI $6.00 below batch; APV ≥$3 est.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>SNP lot (~3 drums/week)</t>
+        </is>
+      </c>
+      <c r="C17" s="51" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D17" s="67" t="n">
+        <v>0.9902354927869617</v>
+      </c>
+      <c r="E17" s="67" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F17" s="67" t="n">
+        <v>3.093818054556199</v>
+      </c>
+      <c r="G17" s="52" t="inlineStr">
+        <is>
+          <t>SNP $0.75 delivered</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>5-drum batch</t>
+        </is>
+      </c>
+      <c r="C18" s="51" t="n">
+        <v>2250</v>
+      </c>
+      <c r="D18" s="67" t="n">
+        <v>0.8517189241626537</v>
+      </c>
+      <c r="E18" s="67" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F18" s="67" t="n">
+        <v>2.909428201514443</v>
+      </c>
+      <c r="G18" s="52" t="inlineStr">
+        <is>
+          <t>PCI $3.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>50 drums</t>
+        </is>
+      </c>
+      <c r="C19" s="51" t="n">
+        <v>22500</v>
+      </c>
+      <c r="D19" s="67" t="n">
+        <v>0.4318278751553078</v>
+      </c>
+      <c r="E19" s="67" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F19" s="67" t="n">
+        <v>2.205532239477101</v>
+      </c>
+      <c r="G19" s="52" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>150 drums (a year)</t>
+        </is>
+      </c>
+      <c r="C20" s="51" t="n">
+        <v>67600</v>
+      </c>
+      <c r="D20" s="67" t="n">
+        <v>0.3121598974418646</v>
+      </c>
+      <c r="E20" s="67" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F20" s="67" t="n">
+        <v>1.9321513147772</v>
+      </c>
+      <c r="G20" s="52" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6892,7 +7396,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7129,7 +7633,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7532,7 +8036,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7905,197 +8409,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B2:G10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="2">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>If SNP Inc. raises price on the volume it keeps (Year 1, PCI quote $3.50, 50 drums to PCI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Losing a third of our volume may cost SNP its batch efficiency. A surcharge on the retained ~2/3 compounds the premium.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>SNP surcharge</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>SNP $/lb</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>SNP annual (retained)</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>PCI annual</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Premium vs today</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="21">
-        <f>SNPlb*(1+B6)</f>
-        <v/>
-      </c>
-      <c r="D6" s="15">
-        <f>LbWk*Weeks*(1-EffShare)*C6</f>
-        <v/>
-      </c>
-      <c r="E6" s="15">
-        <f>LbWk*Weeks*EffShare*PCImid</f>
-        <v/>
-      </c>
-      <c r="F6" s="15">
-        <f>D6+E6</f>
-        <v/>
-      </c>
-      <c r="G6" s="15">
-        <f>F6-LbWk*Weeks*SNPlb</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="24" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C7" s="21">
-        <f>SNPlb*(1+B7)</f>
-        <v/>
-      </c>
-      <c r="D7" s="15">
-        <f>LbWk*Weeks*(1-EffShare)*C7</f>
-        <v/>
-      </c>
-      <c r="E7" s="15">
-        <f>LbWk*Weeks*EffShare*PCImid</f>
-        <v/>
-      </c>
-      <c r="F7" s="15">
-        <f>D7+E7</f>
-        <v/>
-      </c>
-      <c r="G7" s="15">
-        <f>F7-LbWk*Weeks*SNPlb</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="24" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C8" s="21">
-        <f>SNPlb*(1+B8)</f>
-        <v/>
-      </c>
-      <c r="D8" s="15">
-        <f>LbWk*Weeks*(1-EffShare)*C8</f>
-        <v/>
-      </c>
-      <c r="E8" s="15">
-        <f>LbWk*Weeks*EffShare*PCImid</f>
-        <v/>
-      </c>
-      <c r="F8" s="15">
-        <f>D8+E8</f>
-        <v/>
-      </c>
-      <c r="G8" s="15">
-        <f>F8-LbWk*Weeks*SNPlb</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="24" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C9" s="21">
-        <f>SNPlb*(1+B9)</f>
-        <v/>
-      </c>
-      <c r="D9" s="15">
-        <f>LbWk*Weeks*(1-EffShare)*C9</f>
-        <v/>
-      </c>
-      <c r="E9" s="15">
-        <f>LbWk*Weeks*EffShare*PCImid</f>
-        <v/>
-      </c>
-      <c r="F9" s="15">
-        <f>D9+E9</f>
-        <v/>
-      </c>
-      <c r="G9" s="15">
-        <f>F9-LbWk*Weeks*SNPlb</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="24" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="C10" s="21">
-        <f>SNPlb*(1+B10)</f>
-        <v/>
-      </c>
-      <c r="D10" s="15">
-        <f>LbWk*Weeks*(1-EffShare)*C10</f>
-        <v/>
-      </c>
-      <c r="E10" s="15">
-        <f>LbWk*Weeks*EffShare*PCImid</f>
-        <v/>
-      </c>
-      <c r="F10" s="15">
-        <f>D10+E10</f>
-        <v/>
-      </c>
-      <c r="G10" s="15">
-        <f>F10-LbWk*Weeks*SNPlb</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Workbook: fix column references (Summary premium/break-even, block-rotation rows, Options premium) and a note read as a formula
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
@@ -826,7 +826,7 @@
         </is>
       </c>
       <c r="C13" s="55">
-        <f>B12-B10</f>
+        <f>C12-C10</f>
         <v/>
       </c>
       <c r="D13" s="56" t="inlineStr">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="C14" s="57">
-        <f>B13/B10</f>
+        <f>C13/C10</f>
         <v/>
       </c>
       <c r="D14" s="52" t="inlineStr">
@@ -906,7 +906,7 @@
         </is>
       </c>
       <c r="C18" s="54">
-        <f>B13/0.10</f>
+        <f>C13/0.10</f>
         <v/>
       </c>
       <c r="D18" s="52" t="inlineStr">
@@ -922,7 +922,7 @@
         </is>
       </c>
       <c r="C19" s="54">
-        <f>B13/0.05</f>
+        <f>C13/0.05</f>
         <v/>
       </c>
       <c r="D19" s="52" t="inlineStr">
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="C20" s="54">
-        <f>B13/0.02</f>
+        <f>C13/0.02</f>
         <v/>
       </c>
       <c r="D20" s="52" t="inlineStr">
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>B6-LbWk*Weeks*SNPlb</f>
+        <f>C6-LbWk*Weeks*SNPlb</f>
         <v/>
       </c>
       <c r="D7" s="30" t="inlineStr">
@@ -1847,9 +1847,10 @@
         <f>PCIq</f>
         <v/>
       </c>
-      <c r="D16" s="2">
-        <f> the real quote (row 27). Every 'MID' figure in the legacy tabs now uses $3.50.</f>
-        <v/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Points to the real quote (row 27). Every 'MID' figure in the legacy tabs now uses $3.50.</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -7227,7 +7228,7 @@
         </is>
       </c>
       <c r="C29" s="48">
-        <f>B28/(LbWk/7)</f>
+        <f>C28/(LbWk/7)</f>
         <v/>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -7243,7 +7244,7 @@
         </is>
       </c>
       <c r="C30" s="48">
-        <f>B28/(LbWk/3)</f>
+        <f>C28/(LbWk/3)</f>
         <v/>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -7259,7 +7260,7 @@
         </is>
       </c>
       <c r="C31" s="48">
-        <f>B30-B28/LbWk</f>
+        <f>C30-C28/LbWk</f>
         <v/>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -7290,7 +7291,7 @@
         </is>
       </c>
       <c r="C33" s="48">
-        <f>18-B32</f>
+        <f>18-C32</f>
         <v/>
       </c>
       <c r="D33" s="2" t="inlineStr"/>
@@ -7302,7 +7303,7 @@
         </is>
       </c>
       <c r="C34" s="48">
-        <f>B33-B29</f>
+        <f>C33-C29</f>
         <v/>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -7318,7 +7319,7 @@
         </is>
       </c>
       <c r="C35" s="48">
-        <f>B28/(LbWk*2/3/7)</f>
+        <f>C28/(LbWk*2/3/7)</f>
         <v/>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -7334,7 +7335,7 @@
         </is>
       </c>
       <c r="C36" s="48">
-        <f>B28/(LbWk/3/7)</f>
+        <f>C28/(LbWk/3/7)</f>
         <v/>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -7350,7 +7351,7 @@
         </is>
       </c>
       <c r="C37" s="24">
-        <f>B28/((30-B32)*LbWk/7)</f>
+        <f>C28/((30-C32)*LbWk/7)</f>
         <v/>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -7366,7 +7367,7 @@
         </is>
       </c>
       <c r="C38" s="15">
-        <f>B28*PCIq</f>
+        <f>C28*PCIq</f>
         <v/>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -7382,7 +7383,7 @@
         </is>
       </c>
       <c r="C39" s="15">
-        <f>B28*(PCIq-SNPlb)</f>
+        <f>C28*(PCIq-SNPlb)</f>
         <v/>
       </c>
       <c r="D39" s="2" t="inlineStr">

</xml_diff>

<commit_message>
New slide: blended cost per lb of PVA with 1/2/3 PCI batches a year; matching Summary rows in the workbook
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Supplier_Leadership_Model.xlsx
@@ -50,7 +50,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
@@ -58,6 +58,7 @@
     <numFmt numFmtId="168" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="169" formatCode="0.0"/>
     <numFmt numFmtId="170" formatCode="0.000"/>
+    <numFmt numFmtId="171" formatCode="&quot;$&quot;0.000"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -189,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -303,6 +304,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="171" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -668,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D29"/>
+  <dimension ref="B2:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="2" max="2"/>
@@ -1078,14 +1080,94 @@
     <row r="29">
       <c r="B29" s="11" t="inlineStr">
         <is>
+          <t>Blended $/lb, all our PVA — today</t>
+        </is>
+      </c>
+      <c r="C29" s="71">
+        <f>C10/C6</f>
+        <v/>
+      </c>
+      <c r="D29" s="52" t="inlineStr">
+        <is>
+          <t>Blended-cost slide</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Blended $/lb — 1 PCI batch a year</t>
+        </is>
+      </c>
+      <c r="C30" s="71">
+        <f>((C6-PCIbatch*DrumLb)*SNPlb+PCIbatch*DrumLb*PCIq)/C6</f>
+        <v/>
+      </c>
+      <c r="D30" s="52" t="inlineStr">
+        <is>
+          <t>Blended-cost slide</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Blended $/lb — 2 PCI batches a year</t>
+        </is>
+      </c>
+      <c r="C31" s="71">
+        <f>((C6-2*PCIbatch*DrumLb)*SNPlb+2*PCIbatch*DrumLb*PCIq)/C6</f>
+        <v/>
+      </c>
+      <c r="D31" s="52" t="inlineStr">
+        <is>
+          <t>Blended-cost slide</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Blended $/lb — 3 PCI batches a year</t>
+        </is>
+      </c>
+      <c r="C32" s="71">
+        <f>((C6-3*PCIbatch*DrumLb)*SNPlb+3*PCIbatch*DrumLb*PCIq)/C6</f>
+        <v/>
+      </c>
+      <c r="D32" s="52" t="inlineStr">
+        <is>
+          <t>Blended-cost slide</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Blended $/lb — Option 1 (one-third from PCI)</t>
+        </is>
+      </c>
+      <c r="C33" s="71">
+        <f>C12/C6</f>
+        <v/>
+      </c>
+      <c r="D33" s="52" t="inlineStr">
+        <is>
+          <t>Blended-cost slide</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="11" t="inlineStr">
+        <is>
           <t>Option 3 — share of volume at 1 / 2 batches</t>
         </is>
       </c>
-      <c r="C29" s="52">
+      <c r="C34" s="52">
         <f>TEXT(PCIbatch*DrumLb/(LbWk*Weeks),"0.0%")&amp;" / "&amp;TEXT(2*PCIbatch*DrumLb/(LbWk*Weeks),"0.0%")</f>
         <v/>
       </c>
-      <c r="D29" s="52" t="inlineStr">
+      <c r="D34" s="52" t="inlineStr">
         <is>
           <t>Options slide</t>
         </is>

</xml_diff>